<commit_message>
feat(prospeccion): las 30 previews de marca, servidas desde presupuestos.nico-soto.es
Las demos por lead son el proyecto Lovable "Home Estimator" (reform-wizard,
4e13bf62), que ya tenía la ruta `demo.$slug`: resuelve la empresa por slug en su
tabla `organizations` y lanza notFound() si no está. El 404 no era la ruta: era
que solo existían dos filas (`simulador` y `reformas-valencia-myj-8f21`, con un
sufijo que no casa con el slug de los mensajes).

Insertadas las 30 empresas con su nombre, logo_url y sus dos colores, sacados de
app/src/demo/brands.ts. Verificado: las 30 dan 200 y el title lleva el nombre de
cada empresa.

CSVs, cola HTML y Excel vuelven a presupuestos.nico-soto.es, que es el dominio
del producto.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -546,43 +546,29 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>AVISO - enlace de la demo corregido</t>
+          <t>Enlace de la demo</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Los CSV del repo apuntan a https://presupuestos.nico-soto.es/demo/&lt;slug&gt;, que hoy devuelve 404</t>
+          <t>Cada lead tiene su preview de marca en https://presupuestos.nico-soto.es/demo/&lt;slug&gt;,</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>(ese subdominio resuelve a 185.158.133.1, no a Vercel; solo su raiz responde 200).</t>
+          <t>con su logo y sus colores. Verificado: las 30 responden 200.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>En este Excel el enlace ya esta corregido a https://www.nico-soto.es/demo/&lt;slug&gt;, que responde 200,</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
-        <is>
-          <t>tanto en la columna 'Demo (URL)' como dentro del texto del mensaje. Los 30 slugs existen en app/src/demo/brands.ts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
         <is>
           <t>Lead 25 (REFORMSPEED) no tiene email: solo contacto por formulario web.</t>
         </is>
@@ -701,12 +687,12 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/reformas-valencia-myj</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-valencia-myj</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>He visto que ofrecéis "Presupuesto Online", pero al final el cliente os deja sus datos y un mensaje. Cada solicitud que os llega todavía os obliga a trabajar antes de saber si merece la pena: entender metros, estancias, alcance, presupuesto... He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada: https://www.nico-soto.es/demo/reformas-valencia-myj</t>
+          <t>He visto que ofrecéis "Presupuesto Online", pero al final el cliente os deja sus datos y un mensaje. Cada solicitud que os llega todavía os obliga a trabajar antes de saber si merece la pena: entender metros, estancias, alcance, presupuesto... He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada: https://presupuestos.nico-soto.es/demo/reformas-valencia-myj</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr"/>
@@ -742,12 +728,12 @@
       </c>
       <c r="G3" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/grupodmh</t>
+          <t>https://presupuestos.nico-soto.es/demo/grupodmh</t>
         </is>
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>Con más de 130 reseñas, imagino que solicitudes no os faltan. Me llamó la atención que sigan entrando básicamente como nombre, teléfono y mensaje. Eso significa que cada lead todavía os obliga a averiguar metros, estancias, alcance y presupuesto antes de saber si merece la pena. Os he montado una demo para enseñaros otra forma de recibirlas: https://www.nico-soto.es/demo/grupodmh</t>
+          <t>Con más de 130 reseñas, imagino que solicitudes no os faltan. Me llamó la atención que sigan entrando básicamente como nombre, teléfono y mensaje. Eso significa que cada lead todavía os obliga a averiguar metros, estancias, alcance y presupuesto antes de saber si merece la pena. Os he montado una demo para enseñaros otra forma de recibirlas: https://presupuestos.nico-soto.es/demo/grupodmh</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr"/>
@@ -783,12 +769,12 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/nou-cabanyal</t>
+          <t>https://presupuestos.nico-soto.es/demo/nou-cabanyal</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>He visto que estáis muy centrados en reforma integral de vivienda, pero la solicitud de presupuesto prácticamente no recoge información sobre la propia vivienda. Al final cada solicitud os obliga a empezar después preguntando lo básico antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado: https://www.nico-soto.es/demo/nou-cabanyal</t>
+          <t>He visto que estáis muy centrados en reforma integral de vivienda, pero la solicitud de presupuesto prácticamente no recoge información sobre la propia vivienda. Al final cada solicitud os obliga a empezar después preguntando lo básico antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado: https://presupuestos.nico-soto.es/demo/nou-cabanyal</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr"/>
@@ -824,12 +810,12 @@
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/reformas-lujan</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-lujan</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>Tenéis unas 130 reseñas, pero cuando alguien pide información la web recoge poco más que nombre, email y mensaje. Cada solicitud que entra todavía os obliga a reconstruir el proyecto después antes de saber si realmente merece la pena presupuestarlo. He preparado una demo para enseñaros cómo podría llegaros ya cualificado: https://www.nico-soto.es/demo/reformas-lujan</t>
+          <t>Tenéis unas 130 reseñas, pero cuando alguien pide información la web recoge poco más que nombre, email y mensaje. Cada solicitud que entra todavía os obliga a reconstruir el proyecto después antes de saber si realmente merece la pena presupuestarlo. He preparado una demo para enseñaros cómo podría llegaros ya cualificado: https://presupuestos.nico-soto.es/demo/reformas-lujan</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr"/>
@@ -865,12 +851,12 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/reformas-claiz</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-claiz</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Me llamó la atención que, teniendo 5 estrellas y casi 90 reseñas, la petición de presupuesto se reduzca prácticamente a tres campos. El trabajo de entender la reforma empieza cuando ya ha llegado el lead. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada solicitud con metros, estancias, fotos, timing y presupuesto ya recogidos: https://www.nico-soto.es/demo/reformas-claiz</t>
+          <t>Me llamó la atención que, teniendo 5 estrellas y casi 90 reseñas, la petición de presupuesto se reduzca prácticamente a tres campos. El trabajo de entender la reforma empieza cuando ya ha llegado el lead. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada solicitud con metros, estancias, fotos, timing y presupuesto ya recogidos: https://presupuestos.nico-soto.es/demo/reformas-claiz</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr"/>
@@ -906,12 +892,12 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/geteco</t>
+          <t>https://presupuestos.nico-soto.es/demo/geteco</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>He visto que trabajáis reformas de pisos, chalets y casas, pero cuando alguien pide presupuesto la web no distingue prácticamente nada de eso. Cada solicitud os obliga después a averiguar qué quiere realmente el cliente antes de saber si merece la pena. He montado una demo sobre vuestra propia marca para enseñaros cómo podría funcionar: https://www.nico-soto.es/demo/geteco</t>
+          <t>He visto que trabajáis reformas de pisos, chalets y casas, pero cuando alguien pide presupuesto la web no distingue prácticamente nada de eso. Cada solicitud os obliga después a averiguar qué quiere realmente el cliente antes de saber si merece la pena. He montado una demo sobre vuestra propia marca para enseñaros cómo podría funcionar: https://presupuestos.nico-soto.es/demo/geteco</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr"/>
@@ -947,12 +933,12 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/reformas-rocha</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-rocha</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Vuestra solicitud ya pregunta cuándo quiere empezar el cliente, que es más de lo que hace casi todo el sector. Pero todavía os falta saber qué quiere reformar, cuántos metros, qué alcance tiene o qué inversión maneja. Es decir: cada solicitud todavía exige trabajo antes de saber si merece la pena. Os he preparado una demo de cómo completaría ese proceso: https://www.nico-soto.es/demo/reformas-rocha</t>
+          <t>Vuestra solicitud ya pregunta cuándo quiere empezar el cliente, que es más de lo que hace casi todo el sector. Pero todavía os falta saber qué quiere reformar, cuántos metros, qué alcance tiene o qué inversión maneja. Es decir: cada solicitud todavía exige trabajo antes de saber si merece la pena. Os he preparado una demo de cómo completaría ese proceso: https://presupuestos.nico-soto.es/demo/reformas-rocha</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
@@ -988,12 +974,12 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/tas-obras-y-reformas</t>
+          <t>https://presupuestos.nico-soto.es/demo/tas-obras-y-reformas</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>He visto que prácticamente todo el contacto entra por WhatsApp o teléfono. Eso hace que cada nueva reforma empiece siempre igual: preguntar qué quiere hacer, metros, estancias, fotos, presupuesto... antes de saber siquiera si merece la pena. He montado una demo para que todo eso pueda llegaros recogido antes de empezar la conversación: https://www.nico-soto.es/demo/tas-obras-y-reformas</t>
+          <t>He visto que prácticamente todo el contacto entra por WhatsApp o teléfono. Eso hace que cada nueva reforma empiece siempre igual: preguntar qué quiere hacer, metros, estancias, fotos, presupuesto... antes de saber siquiera si merece la pena. He montado una demo para que todo eso pueda llegaros recogido antes de empezar la conversación: https://presupuestos.nico-soto.es/demo/tas-obras-y-reformas</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr"/>
@@ -1029,12 +1015,12 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/robles-home</t>
+          <t>https://presupuestos.nico-soto.es/demo/robles-home</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Me ha sorprendido que para una empresa centrada en reformas integrales, la solicitud online recoja prácticamente solo el email. Cada nuevo proyecto empieza entonces con vosotros pidiendo toda la información desde cero. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada: https://www.nico-soto.es/demo/robles-home</t>
+          <t>Me ha sorprendido que para una empresa centrada en reformas integrales, la solicitud online recoja prácticamente solo el email. Cada nuevo proyecto empieza entonces con vosotros pidiendo toda la información desde cero. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada: https://presupuestos.nico-soto.es/demo/robles-home</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
@@ -1070,12 +1056,12 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/marcos-mym</t>
+          <t>https://presupuestos.nico-soto.es/demo/marcos-mym</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>He visto que al cliente básicamente le pedís que "cuente su proyecto" en un campo de texto. El problema es que luego sois vosotros quienes tenéis que traducir ese mensaje a metros, estancias, trabajos y presupuesto antes de saber si merece la pena. He preparado una demo para enseñaros cómo estructuraría ese paso automáticamente: https://www.nico-soto.es/demo/marcos-mym</t>
+          <t>He visto que al cliente básicamente le pedís que "cuente su proyecto" en un campo de texto. El problema es que luego sois vosotros quienes tenéis que traducir ese mensaje a metros, estancias, trabajos y presupuesto antes de saber si merece la pena. He preparado una demo para enseñaros cómo estructuraría ese paso automáticamente: https://presupuestos.nico-soto.es/demo/marcos-mym</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr"/>
@@ -1111,12 +1097,12 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/rfc-reformas</t>
+          <t>https://presupuestos.nico-soto.es/demo/rfc-reformas</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>He visto vuestra página de "Solicita presupuesto gratis". Recogéis el código postal y qué tipo de reforma quiere, pero todavía queda prácticamente todo por averiguar después. Cada solicitud sigue requiriendo trabajo antes de saber si merece la pena. He montado una demo para enseñaros cómo podría llegaros ya completa: https://www.nico-soto.es/demo/rfc-reformas</t>
+          <t>He visto vuestra página de "Solicita presupuesto gratis". Recogéis el código postal y qué tipo de reforma quiere, pero todavía queda prácticamente todo por averiguar después. Cada solicitud sigue requiriendo trabajo antes de saber si merece la pena. He montado una demo para enseñaros cómo podría llegaros ya completa: https://presupuestos.nico-soto.es/demo/rfc-reformas</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
@@ -1152,12 +1138,12 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/metrocuadrado</t>
+          <t>https://presupuestos.nico-soto.es/demo/metrocuadrado</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Me gustó vuestro enfoque de hacer que una reforma sea un proceso más sencillo, pero el primer contacto sigue dependiendo de que el cliente explique en texto libre lo que necesita. Al final sois vosotros quienes tenéis que ordenar toda esa información después. He montado una demo para enseñaros cómo podría llegaros cada proyecto ya estructurado: https://www.nico-soto.es/demo/metrocuadrado</t>
+          <t>Me gustó vuestro enfoque de hacer que una reforma sea un proceso más sencillo, pero el primer contacto sigue dependiendo de que el cliente explique en texto libre lo que necesita. Al final sois vosotros quienes tenéis que ordenar toda esa información después. He montado una demo para enseñaros cómo podría llegaros cada proyecto ya estructurado: https://presupuestos.nico-soto.es/demo/metrocuadrado</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr"/>
@@ -1193,12 +1179,12 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/efenval</t>
+          <t>https://presupuestos.nico-soto.es/demo/efenval</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>He visto que vuestra solicitud acaba dependiendo de que el cliente os cuente lo que necesita. El problema es que ese mensaje todavía hay que convertirlo después en metros, estancias, alcance, fotos y presupuesto para saber si el proyecto merece la pena. He preparado una demo con vuestra marca para enseñaros otra forma de hacerlo: https://www.nico-soto.es/demo/efenval</t>
+          <t>He visto que vuestra solicitud acaba dependiendo de que el cliente os cuente lo que necesita. El problema es que ese mensaje todavía hay que convertirlo después en metros, estancias, alcance, fotos y presupuesto para saber si el proyecto merece la pena. He preparado una demo con vuestra marca para enseñaros otra forma de hacerlo: https://presupuestos.nico-soto.es/demo/efenval</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
@@ -1234,12 +1220,12 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/rdg-reformas</t>
+          <t>https://presupuestos.nico-soto.es/demo/rdg-reformas</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Ofrecéis presupuesto sin compromiso, pero hasta saber si el proyecto merece la pena el compromiso de tiempo lo asumís vosotros: llamadas, preguntas, mediciones, posible visita y preparación del presupuesto. He montado una demo para enseñaros cómo filtrar y entender mucho mejor el proyecto antes de dedicarle ese tiempo: https://www.nico-soto.es/demo/rdg-reformas</t>
+          <t>Ofrecéis presupuesto sin compromiso, pero hasta saber si el proyecto merece la pena el compromiso de tiempo lo asumís vosotros: llamadas, preguntas, mediciones, posible visita y preparación del presupuesto. He montado una demo para enseñaros cómo filtrar y entender mucho mejor el proyecto antes de dedicarle ese tiempo: https://presupuestos.nico-soto.es/demo/rdg-reformas</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr"/>
@@ -1275,12 +1261,12 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/reformas-turia</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-turia</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>He visto que ya dejáis elegir el tipo de reforma, pero después todavía hay que preguntar metros, estancias, alcance, fotos, timing y presupuesto. Es decir, cada solicitud os sigue obligando a trabajar antes de saber si realmente merece la pena. He preparado una demo para enseñaros cómo podría llegaros todo eso ya recogido: https://www.nico-soto.es/demo/reformas-turia</t>
+          <t>He visto que ya dejáis elegir el tipo de reforma, pero después todavía hay que preguntar metros, estancias, alcance, fotos, timing y presupuesto. Es decir, cada solicitud os sigue obligando a trabajar antes de saber si realmente merece la pena. He preparado una demo para enseñaros cómo podría llegaros todo eso ya recogido: https://presupuestos.nico-soto.es/demo/reformas-turia</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr"/>
@@ -1463,12 +1449,12 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/gabi-reformas</t>
+          <t>https://presupuestos.nico-soto.es/demo/gabi-reformas</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>He visto que ofrecéis presupuesto sin compromiso, pero la solicitud os llega básicamente con nombre, email y un mensaje. Al final el compromiso de tiempo empieza después: entender la reforma, metros, alcance, inversión y decidir si merece la pena. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada reforma ya explicada: https://www.nico-soto.es/demo/gabi-reformas</t>
+          <t>He visto que ofrecéis presupuesto sin compromiso, pero la solicitud os llega básicamente con nombre, email y un mensaje. Al final el compromiso de tiempo empieza después: entender la reforma, metros, alcance, inversión y decidir si merece la pena. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada reforma ya explicada: https://presupuestos.nico-soto.es/demo/gabi-reformas</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr"/>
@@ -1504,12 +1490,12 @@
       </c>
       <c r="G3" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/reformas-bailen</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-bailen</t>
         </is>
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>He visto vuestro “solicita tu presupuesto gratis”, pero el formulario recoge nombre, email y mensaje. Cada solicitud todavía os obliga a hacer preguntas y entender el proyecto antes de saber si merece la pena presupuestarlo. He preparado una demo para enseñaros cómo podría llegaros ya cualificado: https://www.nico-soto.es/demo/reformas-bailen</t>
+          <t>He visto vuestro “solicita tu presupuesto gratis”, pero el formulario recoge nombre, email y mensaje. Cada solicitud todavía os obliga a hacer preguntas y entender el proyecto antes de saber si merece la pena presupuestarlo. He preparado una demo para enseñaros cómo podría llegaros ya cualificado: https://presupuestos.nico-soto.es/demo/reformas-bailen</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr"/>
@@ -1545,12 +1531,12 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/grupo-g-reformas</t>
+          <t>https://presupuestos.nico-soto.es/demo/grupo-g-reformas</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Ya preguntáis el tipo de reforma, pero después el cliente tiene que describir el resto en texto libre. Ahí puede caber desde cambiar un baño hasta una integral de 120 m². Cada solicitud todavía requiere trabajo antes de saber si merece la pena. Os he montado una demo de cómo recoger todo eso antes de que llegue el lead: https://www.nico-soto.es/demo/grupo-g-reformas</t>
+          <t>Ya preguntáis el tipo de reforma, pero después el cliente tiene que describir el resto en texto libre. Ahí puede caber desde cambiar un baño hasta una integral de 120 m². Cada solicitud todavía requiere trabajo antes de saber si merece la pena. Os he montado una demo de cómo recoger todo eso antes de que llegue el lead: https://presupuestos.nico-soto.es/demo/grupo-g-reformas</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr"/>
@@ -1586,12 +1572,12 @@
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/azahar-reformas</t>
+          <t>https://presupuestos.nico-soto.es/demo/azahar-reformas</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>He visto que vuestra solicitud recoge nombre, teléfono, email y “¿en qué podemos ayudarte?”. Es decir, prácticamente todo el trabajo de entender la reforma empieza después de recibir el lead. He montado una demo con vuestra marca para que cada solicitud os llegue con el proyecto mucho más claro antes de dedicarle tiempo: https://www.nico-soto.es/demo/azahar-reformas</t>
+          <t>He visto que vuestra solicitud recoge nombre, teléfono, email y “¿en qué podemos ayudarte?”. Es decir, prácticamente todo el trabajo de entender la reforma empieza después de recibir el lead. He montado una demo con vuestra marca para que cada solicitud os llegue con el proyecto mucho más claro antes de dedicarle tiempo: https://presupuestos.nico-soto.es/demo/azahar-reformas</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr"/>
@@ -1627,12 +1613,12 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/todo-reformas-valencia</t>
+          <t>https://presupuestos.nico-soto.es/demo/todo-reformas-valencia</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Me llamó la atención que os posicionéis para búsquedas de presupuesto de reforma de piso en Valencia, pero cuando llega el cliente el formulario apenas recoge sus datos y un mensaje. Cada solicitud todavía os obliga a reconstruir el proyecto antes de saber si merece la pena. He preparado una demo de cómo podría funcionar ese paso: https://www.nico-soto.es/demo/todo-reformas-valencia</t>
+          <t>Me llamó la atención que os posicionéis para búsquedas de presupuesto de reforma de piso en Valencia, pero cuando llega el cliente el formulario apenas recoge sus datos y un mensaje. Cada solicitud todavía os obliga a reconstruir el proyecto antes de saber si merece la pena. He preparado una demo de cómo podría funcionar ese paso: https://presupuestos.nico-soto.es/demo/todo-reformas-valencia</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr"/>
@@ -1668,12 +1654,12 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/reformas-orcu</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-orcu</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>Hacéis reformas integrales, cocinas y baños, pero el cliente tiene que explicar lo que quiere prácticamente desde cero en un mensaje. Luego sois vosotros quienes convertís eso en metros, estancias, trabajos e inversión. He montado una demo para enseñaros cómo podría llegaros esa información ya estructurada: https://www.nico-soto.es/demo/reformas-orcu</t>
+          <t>Hacéis reformas integrales, cocinas y baños, pero el cliente tiene que explicar lo que quiere prácticamente desde cero en un mensaje. Luego sois vosotros quienes convertís eso en metros, estancias, trabajos e inversión. He montado una demo para enseñaros cómo podría llegaros esa información ya estructurada: https://presupuestos.nico-soto.es/demo/reformas-orcu</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr"/>
@@ -1709,12 +1695,12 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/obras-vip</t>
+          <t>https://presupuestos.nico-soto.es/demo/obras-vip</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>He visto que vuestro formulario ya pregunta cuándo quiere realizar el trabajo, pero no recoge metros, estancias, alcance ni inversión. Sabéis cuándo quiere empezar, pero todavía tenéis que averiguar casi todo lo demás antes de saber si merece la pena. He preparado una demo para completar justo esa parte: https://www.nico-soto.es/demo/obras-vip</t>
+          <t>He visto que vuestro formulario ya pregunta cuándo quiere realizar el trabajo, pero no recoge metros, estancias, alcance ni inversión. Sabéis cuándo quiere empezar, pero todavía tenéis que averiguar casi todo lo demás antes de saber si merece la pena. He preparado una demo para completar justo esa parte: https://presupuestos.nico-soto.es/demo/obras-vip</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
@@ -1750,12 +1736,12 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/bono-proyectos</t>
+          <t>https://presupuestos.nico-soto.es/demo/bono-proyectos</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>Vendéis proyectos llave en mano, pero cuando alguien pide información entra por un formulario genérico y todavía tenéis que averiguar todo el alcance del proyecto. Cada solicitud os obliga a trabajar antes de saber si encaja realmente. He preparado una demo para enseñaros cómo podría llegaros mucho más definida: https://www.nico-soto.es/demo/bono-proyectos</t>
+          <t>Vendéis proyectos llave en mano, pero cuando alguien pide información entra por un formulario genérico y todavía tenéis que averiguar todo el alcance del proyecto. Cada solicitud os obliga a trabajar antes de saber si encaja realmente. He preparado una demo para enseñaros cómo podría llegaros mucho más definida: https://presupuestos.nico-soto.es/demo/bono-proyectos</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr"/>
@@ -1791,12 +1777,12 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/vga-reformas</t>
+          <t>https://presupuestos.nico-soto.es/demo/vga-reformas</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>He visto que ya preguntáis el tipo de servicio, pero la cualificación se queda ahí: no metros, estancias, timing, fotos ni inversión prevista. Cada solicitud todavía os obliga a completar todo eso después. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado: https://www.nico-soto.es/demo/vga-reformas</t>
+          <t>He visto que ya preguntáis el tipo de servicio, pero la cualificación se queda ahí: no metros, estancias, timing, fotos ni inversión prevista. Cada solicitud todavía os obliga a completar todo eso después. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado: https://presupuestos.nico-soto.es/demo/vga-reformas</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
@@ -1828,12 +1814,12 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/reformspeed</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformspeed</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>Tenéis una página específica para solicitar presupuesto, pero al final el cliente deja sus datos y os cuenta libremente lo que necesita. El trabajo de convertir eso en un proyecto presupuestable sigue siendo vuestro. He preparado una demo para que veáis cómo podría llegaros ya estructurado antes de dedicarle tiempo: https://www.nico-soto.es/demo/reformspeed</t>
+          <t>Tenéis una página específica para solicitar presupuesto, pero al final el cliente deja sus datos y os cuenta libremente lo que necesita. El trabajo de convertir eso en un proyecto presupuestable sigue siendo vuestro. He preparado una demo para que veáis cómo podría llegaros ya estructurado antes de dedicarle tiempo: https://presupuestos.nico-soto.es/demo/reformspeed</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr"/>
@@ -1869,12 +1855,12 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/grupo-expovall</t>
+          <t>https://presupuestos.nico-soto.es/demo/grupo-expovall</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>He visto que la petición de presupuesto os llega básicamente como datos de contacto y un mensaje. Eso significa que cada nuevo lead todavía necesita una conversación para saber qué quiere, cuánto, cuándo y si realmente merece la pena presupuestarlo. He montado una demo para enseñaros cómo podría llegaros esa reforma ya explicada: https://www.nico-soto.es/demo/grupo-expovall</t>
+          <t>He visto que la petición de presupuesto os llega básicamente como datos de contacto y un mensaje. Eso significa que cada nuevo lead todavía necesita una conversación para saber qué quiere, cuánto, cuándo y si realmente merece la pena presupuestarlo. He montado una demo para enseñaros cómo podría llegaros esa reforma ya explicada: https://presupuestos.nico-soto.es/demo/grupo-expovall</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
@@ -1910,12 +1896,12 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/cecever</t>
+          <t>https://presupuestos.nico-soto.es/demo/cecever</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Trabajáis cocinas, baños y reformas de pisos, pero la solicitud online no diferencia entre ninguno de esos proyectos. Cada lead os llega sin la información que determina el trabajo y sois vosotros quienes tenéis que sacársela después. He preparado una demo con vuestra marca para enseñaros otra forma de recibirlos: https://www.nico-soto.es/demo/cecever</t>
+          <t>Trabajáis cocinas, baños y reformas de pisos, pero la solicitud online no diferencia entre ninguno de esos proyectos. Cada lead os llega sin la información que determina el trabajo y sois vosotros quienes tenéis que sacársela después. He preparado una demo con vuestra marca para enseñaros otra forma de recibirlos: https://presupuestos.nico-soto.es/demo/cecever</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr"/>
@@ -1951,12 +1937,12 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/reformas-ferreira</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-ferreira</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>He visto que cuando alguien contacta os deja nombre, teléfono, email y un mensaje. Es decir, todo lo importante sobre la reforma empieza después. Cada solicitud todavía os obliga a trabajar antes de saber si merece la pena. He montado una demo para enseñaros cómo podría llegaros ya cualificada: https://www.nico-soto.es/demo/reformas-ferreira</t>
+          <t>He visto que cuando alguien contacta os deja nombre, teléfono, email y un mensaje. Es decir, todo lo importante sobre la reforma empieza después. Cada solicitud todavía os obliga a trabajar antes de saber si merece la pena. He montado una demo para enseñaros cómo podría llegaros ya cualificada: https://presupuestos.nico-soto.es/demo/reformas-ferreira</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
@@ -1992,12 +1978,12 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/dekorinex</t>
+          <t>https://presupuestos.nico-soto.es/demo/dekorinex</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Tenéis un CTA de “Solicita presupuesto Online”, pero el proceso termina en un formulario de cuatro campos. Online es la solicitud; el trabajo de entender y presupuestar la reforma sigue viniendo después. He preparado una demo para enseñaros cómo convertir ese “presupuesto online” en algo bastante más útil: https://www.nico-soto.es/demo/dekorinex</t>
+          <t>Tenéis un CTA de “Solicita presupuesto Online”, pero el proceso termina en un formulario de cuatro campos. Online es la solicitud; el trabajo de entender y presupuestar la reforma sigue viniendo después. He preparado una demo para enseñaros cómo convertir ese “presupuesto online” en algo bastante más útil: https://presupuestos.nico-soto.es/demo/dekorinex</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr"/>
@@ -2033,12 +2019,12 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>https://www.nico-soto.es/demo/incoval</t>
+          <t>https://presupuestos.nico-soto.es/demo/incoval</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Lleváis años haciendo reformas integrales, cocinas y baños, pero el formulario todavía deja prácticamente todo el proyecto dentro de un mensaje libre. Cada solicitud os obliga a interpretarla y cualificarla antes de saber si merece la pena. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada reforma ya explicada: https://www.nico-soto.es/demo/incoval</t>
+          <t>Lleváis años haciendo reformas integrales, cocinas y baños, pero el formulario todavía deja prácticamente todo el proyecto dentro de un mensaje libre. Cada solicitud os obliga a interpretarla y cualificarla antes de saber si merece la pena. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada reforma ya explicada: https://presupuestos.nico-soto.es/demo/incoval</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
docs(prospeccion): datos de contacto de la ronda en la hoja Léeme
hola@nico-soto.es y el WhatsApp de negocio, que se teclean en cada uno de los 30
formularios.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -568,7 +568,31 @@
       <c r="A9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Datos para rellenar los formularios</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Email de respuesta:  hola@nico-soto.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Telefono / WhatsApp: +34 600 78 22 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Lead 25 (REFORMSPEED) no tiene email: solo contacto por formulario web.</t>
         </is>

</xml_diff>

<commit_message>
feat(prospeccion): saludo y cierre en los 30 mensajes, con la URL aislada
Apertura "Hola, equipo de <marca>:" y cierre "Son solo dos minutos y sin
compromiso.". El nombre del saludo sale de brands.ts, no del CSV: ahí está mejor
escrito ("Reformas Valencia M&J" y no "REFORMAS VALENCIA MyJ"). Dos excepciones a
mano: TAS Obras y Reformas (su capitalizado real parece una errata en un saludo) y
Valltro (se corta el "· Grupo Expovall").

La URL pasa a ir sola en su línea, sin puntuación pegada: se ve más y los clientes
de correo la autoenlazan sin comerse el último carácter.

Los tres soportes a la vez: CSVs, cola HTML (tabla NOMBRES + composición del texto)
y Excel, con la fila más alta porque el mensaje ocupa el triple.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -682,7 +682,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="92" customHeight="1">
+    <row r="2" ht="165" customHeight="1">
       <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
@@ -716,14 +716,17 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>He visto que ofrecéis "Presupuesto Online", pero al final el cliente os deja sus datos y un mensaje. Cada solicitud que os llega todavía os obliga a trabajar antes de saber si merece la pena: entender metros, estancias, alcance, presupuesto... He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada: https://presupuestos.nico-soto.es/demo/reformas-valencia-myj</t>
+          <t>Hola, equipo de Reformas Valencia M&amp;J:
+He visto que ofrecéis "Presupuesto Online", pero al final el cliente os deja sus datos y un mensaje. Cada solicitud que os llega todavía os obliga a trabajar antes de saber si merece la pena: entender metros, estancias, alcance, presupuesto... He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/reformas-valencia-myj
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr"/>
       <c r="J2" s="4" t="inlineStr"/>
       <c r="K2" s="4" t="inlineStr"/>
     </row>
-    <row r="3" ht="92" customHeight="1">
+    <row r="3" ht="165" customHeight="1">
       <c r="A3" s="8" t="n">
         <v>2</v>
       </c>
@@ -757,14 +760,17 @@
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>Con más de 130 reseñas, imagino que solicitudes no os faltan. Me llamó la atención que sigan entrando básicamente como nombre, teléfono y mensaje. Eso significa que cada lead todavía os obliga a averiguar metros, estancias, alcance y presupuesto antes de saber si merece la pena. Os he montado una demo para enseñaros otra forma de recibirlas: https://presupuestos.nico-soto.es/demo/grupodmh</t>
+          <t>Hola, equipo de GrupoDMH Reformas Integrales:
+Con más de 130 reseñas, imagino que solicitudes no os faltan. Me llamó la atención que sigan entrando básicamente como nombre, teléfono y mensaje. Eso significa que cada lead todavía os obliga a averiguar metros, estancias, alcance y presupuesto antes de saber si merece la pena. Os he montado una demo para enseñaros otra forma de recibirlas:
+https://presupuestos.nico-soto.es/demo/grupodmh
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr"/>
       <c r="J3" s="9" t="inlineStr"/>
       <c r="K3" s="9" t="inlineStr"/>
     </row>
-    <row r="4" ht="92" customHeight="1">
+    <row r="4" ht="165" customHeight="1">
       <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
@@ -798,14 +804,17 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>He visto que estáis muy centrados en reforma integral de vivienda, pero la solicitud de presupuesto prácticamente no recoge información sobre la propia vivienda. Al final cada solicitud os obliga a empezar después preguntando lo básico antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado: https://presupuestos.nico-soto.es/demo/nou-cabanyal</t>
+          <t>Hola, equipo de Reformas Nou Cabanyal:
+He visto que estáis muy centrados en reforma integral de vivienda, pero la solicitud de presupuesto prácticamente no recoge información sobre la propia vivienda. Al final cada solicitud os obliga a empezar después preguntando lo básico antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado:
+https://presupuestos.nico-soto.es/demo/nou-cabanyal
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr"/>
       <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr"/>
     </row>
-    <row r="5" ht="92" customHeight="1">
+    <row r="5" ht="165" customHeight="1">
       <c r="A5" s="8" t="n">
         <v>4</v>
       </c>
@@ -839,14 +848,17 @@
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>Tenéis unas 130 reseñas, pero cuando alguien pide información la web recoge poco más que nombre, email y mensaje. Cada solicitud que entra todavía os obliga a reconstruir el proyecto después antes de saber si realmente merece la pena presupuestarlo. He preparado una demo para enseñaros cómo podría llegaros ya cualificado: https://presupuestos.nico-soto.es/demo/reformas-lujan</t>
+          <t>Hola, equipo de Reformas Luján:
+Tenéis unas 130 reseñas, pero cuando alguien pide información la web recoge poco más que nombre, email y mensaje. Cada solicitud que entra todavía os obliga a reconstruir el proyecto después antes de saber si realmente merece la pena presupuestarlo. He preparado una demo para enseñaros cómo podría llegaros ya cualificado:
+https://presupuestos.nico-soto.es/demo/reformas-lujan
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr"/>
       <c r="J5" s="9" t="inlineStr"/>
       <c r="K5" s="9" t="inlineStr"/>
     </row>
-    <row r="6" ht="92" customHeight="1">
+    <row r="6" ht="165" customHeight="1">
       <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
@@ -880,14 +892,17 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Me llamó la atención que, teniendo 5 estrellas y casi 90 reseñas, la petición de presupuesto se reduzca prácticamente a tres campos. El trabajo de entender la reforma empieza cuando ya ha llegado el lead. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada solicitud con metros, estancias, fotos, timing y presupuesto ya recogidos: https://presupuestos.nico-soto.es/demo/reformas-claiz</t>
+          <t>Hola, equipo de Reformas Claiz:
+Me llamó la atención que, teniendo 5 estrellas y casi 90 reseñas, la petición de presupuesto se reduzca prácticamente a tres campos. El trabajo de entender la reforma empieza cuando ya ha llegado el lead. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada solicitud con metros, estancias, fotos, timing y presupuesto ya recogidos:
+https://presupuestos.nico-soto.es/demo/reformas-claiz
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr"/>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="4" t="inlineStr"/>
     </row>
-    <row r="7" ht="92" customHeight="1">
+    <row r="7" ht="165" customHeight="1">
       <c r="A7" s="8" t="n">
         <v>6</v>
       </c>
@@ -921,14 +936,17 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>He visto que trabajáis reformas de pisos, chalets y casas, pero cuando alguien pide presupuesto la web no distingue prácticamente nada de eso. Cada solicitud os obliga después a averiguar qué quiere realmente el cliente antes de saber si merece la pena. He montado una demo sobre vuestra propia marca para enseñaros cómo podría funcionar: https://presupuestos.nico-soto.es/demo/geteco</t>
+          <t>Hola, equipo de GETECO:
+He visto que trabajáis reformas de pisos, chalets y casas, pero cuando alguien pide presupuesto la web no distingue prácticamente nada de eso. Cada solicitud os obliga después a averiguar qué quiere realmente el cliente antes de saber si merece la pena. He montado una demo sobre vuestra propia marca para enseñaros cómo podría funcionar:
+https://presupuestos.nico-soto.es/demo/geteco
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr"/>
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="9" t="inlineStr"/>
     </row>
-    <row r="8" ht="92" customHeight="1">
+    <row r="8" ht="165" customHeight="1">
       <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
@@ -962,14 +980,17 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Vuestra solicitud ya pregunta cuándo quiere empezar el cliente, que es más de lo que hace casi todo el sector. Pero todavía os falta saber qué quiere reformar, cuántos metros, qué alcance tiene o qué inversión maneja. Es decir: cada solicitud todavía exige trabajo antes de saber si merece la pena. Os he preparado una demo de cómo completaría ese proceso: https://presupuestos.nico-soto.es/demo/reformas-rocha</t>
+          <t>Hola, equipo de Reformas Rocha:
+Vuestra solicitud ya pregunta cuándo quiere empezar el cliente, que es más de lo que hace casi todo el sector. Pero todavía os falta saber qué quiere reformar, cuántos metros, qué alcance tiene o qué inversión maneja. Es decir: cada solicitud todavía exige trabajo antes de saber si merece la pena. Os he preparado una demo de cómo completaría ese proceso:
+https://presupuestos.nico-soto.es/demo/reformas-rocha
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="4" t="inlineStr"/>
     </row>
-    <row r="9" ht="92" customHeight="1">
+    <row r="9" ht="165" customHeight="1">
       <c r="A9" s="8" t="n">
         <v>8</v>
       </c>
@@ -1003,14 +1024,17 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>He visto que prácticamente todo el contacto entra por WhatsApp o teléfono. Eso hace que cada nueva reforma empiece siempre igual: preguntar qué quiere hacer, metros, estancias, fotos, presupuesto... antes de saber siquiera si merece la pena. He montado una demo para que todo eso pueda llegaros recogido antes de empezar la conversación: https://presupuestos.nico-soto.es/demo/tas-obras-y-reformas</t>
+          <t>Hola, equipo de TAS Obras y Reformas:
+He visto que prácticamente todo el contacto entra por WhatsApp o teléfono. Eso hace que cada nueva reforma empiece siempre igual: preguntar qué quiere hacer, metros, estancias, fotos, presupuesto... antes de saber siquiera si merece la pena. He montado una demo para que todo eso pueda llegaros recogido antes de empezar la conversación:
+https://presupuestos.nico-soto.es/demo/tas-obras-y-reformas
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr"/>
       <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="9" t="inlineStr"/>
     </row>
-    <row r="10" ht="92" customHeight="1">
+    <row r="10" ht="165" customHeight="1">
       <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
@@ -1044,14 +1068,17 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Me ha sorprendido que para una empresa centrada en reformas integrales, la solicitud online recoja prácticamente solo el email. Cada nuevo proyecto empieza entonces con vosotros pidiendo toda la información desde cero. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada: https://presupuestos.nico-soto.es/demo/robles-home</t>
+          <t>Hola, equipo de ROBLES Home:
+Me ha sorprendido que para una empresa centrada en reformas integrales, la solicitud online recoja prácticamente solo el email. Cada nuevo proyecto empieza entonces con vosotros pidiendo toda la información desde cero. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/robles-home
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="4" t="inlineStr"/>
     </row>
-    <row r="11" ht="92" customHeight="1">
+    <row r="11" ht="165" customHeight="1">
       <c r="A11" s="8" t="n">
         <v>10</v>
       </c>
@@ -1085,14 +1112,17 @@
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>He visto que al cliente básicamente le pedís que "cuente su proyecto" en un campo de texto. El problema es que luego sois vosotros quienes tenéis que traducir ese mensaje a metros, estancias, trabajos y presupuesto antes de saber si merece la pena. He preparado una demo para enseñaros cómo estructuraría ese paso automáticamente: https://presupuestos.nico-soto.es/demo/marcos-mym</t>
+          <t>Hola, equipo de Reformas Marcos MyM:
+He visto que al cliente básicamente le pedís que "cuente su proyecto" en un campo de texto. El problema es que luego sois vosotros quienes tenéis que traducir ese mensaje a metros, estancias, trabajos y presupuesto antes de saber si merece la pena. He preparado una demo para enseñaros cómo estructuraría ese paso automáticamente:
+https://presupuestos.nico-soto.es/demo/marcos-mym
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr"/>
       <c r="J11" s="9" t="inlineStr"/>
       <c r="K11" s="9" t="inlineStr"/>
     </row>
-    <row r="12" ht="92" customHeight="1">
+    <row r="12" ht="165" customHeight="1">
       <c r="A12" s="3" t="n">
         <v>11</v>
       </c>
@@ -1126,14 +1156,17 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>He visto vuestra página de "Solicita presupuesto gratis". Recogéis el código postal y qué tipo de reforma quiere, pero todavía queda prácticamente todo por averiguar después. Cada solicitud sigue requiriendo trabajo antes de saber si merece la pena. He montado una demo para enseñaros cómo podría llegaros ya completa: https://presupuestos.nico-soto.es/demo/rfc-reformas</t>
+          <t>Hola, equipo de RFC Reformas:
+He visto vuestra página de "Solicita presupuesto gratis". Recogéis el código postal y qué tipo de reforma quiere, pero todavía queda prácticamente todo por averiguar después. Cada solicitud sigue requiriendo trabajo antes de saber si merece la pena. He montado una demo para enseñaros cómo podría llegaros ya completa:
+https://presupuestos.nico-soto.es/demo/rfc-reformas
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr"/>
     </row>
-    <row r="13" ht="92" customHeight="1">
+    <row r="13" ht="165" customHeight="1">
       <c r="A13" s="8" t="n">
         <v>12</v>
       </c>
@@ -1167,14 +1200,17 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Me gustó vuestro enfoque de hacer que una reforma sea un proceso más sencillo, pero el primer contacto sigue dependiendo de que el cliente explique en texto libre lo que necesita. Al final sois vosotros quienes tenéis que ordenar toda esa información después. He montado una demo para enseñaros cómo podría llegaros cada proyecto ya estructurado: https://presupuestos.nico-soto.es/demo/metrocuadrado</t>
+          <t>Hola, equipo de Metrocuadrado Estudio:
+Me gustó vuestro enfoque de hacer que una reforma sea un proceso más sencillo, pero el primer contacto sigue dependiendo de que el cliente explique en texto libre lo que necesita. Al final sois vosotros quienes tenéis que ordenar toda esa información después. He montado una demo para enseñaros cómo podría llegaros cada proyecto ya estructurado:
+https://presupuestos.nico-soto.es/demo/metrocuadrado
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr"/>
       <c r="J13" s="9" t="inlineStr"/>
       <c r="K13" s="9" t="inlineStr"/>
     </row>
-    <row r="14" ht="92" customHeight="1">
+    <row r="14" ht="165" customHeight="1">
       <c r="A14" s="3" t="n">
         <v>13</v>
       </c>
@@ -1208,14 +1244,17 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>He visto que vuestra solicitud acaba dependiendo de que el cliente os cuente lo que necesita. El problema es que ese mensaje todavía hay que convertirlo después en metros, estancias, alcance, fotos y presupuesto para saber si el proyecto merece la pena. He preparado una demo con vuestra marca para enseñaros otra forma de hacerlo: https://presupuestos.nico-soto.es/demo/efenval</t>
+          <t>Hola, equipo de Construcciones Efenval:
+He visto que vuestra solicitud acaba dependiendo de que el cliente os cuente lo que necesita. El problema es que ese mensaje todavía hay que convertirlo después en metros, estancias, alcance, fotos y presupuesto para saber si el proyecto merece la pena. He preparado una demo con vuestra marca para enseñaros otra forma de hacerlo:
+https://presupuestos.nico-soto.es/demo/efenval
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr"/>
     </row>
-    <row r="15" ht="92" customHeight="1">
+    <row r="15" ht="165" customHeight="1">
       <c r="A15" s="8" t="n">
         <v>14</v>
       </c>
@@ -1249,14 +1288,17 @@
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Ofrecéis presupuesto sin compromiso, pero hasta saber si el proyecto merece la pena el compromiso de tiempo lo asumís vosotros: llamadas, preguntas, mediciones, posible visita y preparación del presupuesto. He montado una demo para enseñaros cómo filtrar y entender mucho mejor el proyecto antes de dedicarle ese tiempo: https://presupuestos.nico-soto.es/demo/rdg-reformas</t>
+          <t>Hola, equipo de RDG Reformas:
+Ofrecéis presupuesto sin compromiso, pero hasta saber si el proyecto merece la pena el compromiso de tiempo lo asumís vosotros: llamadas, preguntas, mediciones, posible visita y preparación del presupuesto. He montado una demo para enseñaros cómo filtrar y entender mucho mejor el proyecto antes de dedicarle ese tiempo:
+https://presupuestos.nico-soto.es/demo/rdg-reformas
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr"/>
       <c r="J15" s="9" t="inlineStr"/>
       <c r="K15" s="9" t="inlineStr"/>
     </row>
-    <row r="16" ht="92" customHeight="1">
+    <row r="16" ht="165" customHeight="1">
       <c r="A16" s="3" t="n">
         <v>15</v>
       </c>
@@ -1290,7 +1332,10 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>He visto que ya dejáis elegir el tipo de reforma, pero después todavía hay que preguntar metros, estancias, alcance, fotos, timing y presupuesto. Es decir, cada solicitud os sigue obligando a trabajar antes de saber si realmente merece la pena. He preparado una demo para enseñaros cómo podría llegaros todo eso ya recogido: https://presupuestos.nico-soto.es/demo/reformas-turia</t>
+          <t>Hola, equipo de Reformas Turia:
+He visto que ya dejáis elegir el tipo de reforma, pero después todavía hay que preguntar metros, estancias, alcance, fotos, timing y presupuesto. Es decir, cada solicitud os sigue obligando a trabajar antes de saber si realmente merece la pena. He preparado una demo para enseñaros cómo podría llegaros todo eso ya recogido:
+https://presupuestos.nico-soto.es/demo/reformas-turia
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr"/>
@@ -1444,7 +1489,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="92" customHeight="1">
+    <row r="2" ht="165" customHeight="1">
       <c r="A2" s="3" t="n">
         <v>16</v>
       </c>
@@ -1478,14 +1523,17 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>He visto que ofrecéis presupuesto sin compromiso, pero la solicitud os llega básicamente con nombre, email y un mensaje. Al final el compromiso de tiempo empieza después: entender la reforma, metros, alcance, inversión y decidir si merece la pena. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada reforma ya explicada: https://presupuestos.nico-soto.es/demo/gabi-reformas</t>
+          <t>Hola, equipo de Gabi Reformas:
+He visto que ofrecéis presupuesto sin compromiso, pero la solicitud os llega básicamente con nombre, email y un mensaje. Al final el compromiso de tiempo empieza después: entender la reforma, metros, alcance, inversión y decidir si merece la pena. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/gabi-reformas
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr"/>
       <c r="J2" s="4" t="inlineStr"/>
       <c r="K2" s="4" t="inlineStr"/>
     </row>
-    <row r="3" ht="92" customHeight="1">
+    <row r="3" ht="165" customHeight="1">
       <c r="A3" s="8" t="n">
         <v>17</v>
       </c>
@@ -1519,14 +1567,17 @@
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>He visto vuestro “solicita tu presupuesto gratis”, pero el formulario recoge nombre, email y mensaje. Cada solicitud todavía os obliga a hacer preguntas y entender el proyecto antes de saber si merece la pena presupuestarlo. He preparado una demo para enseñaros cómo podría llegaros ya cualificado: https://presupuestos.nico-soto.es/demo/reformas-bailen</t>
+          <t>Hola, equipo de Reformas Bailén:
+He visto vuestro “solicita tu presupuesto gratis”, pero el formulario recoge nombre, email y mensaje. Cada solicitud todavía os obliga a hacer preguntas y entender el proyecto antes de saber si merece la pena presupuestarlo. He preparado una demo para enseñaros cómo podría llegaros ya cualificado:
+https://presupuestos.nico-soto.es/demo/reformas-bailen
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr"/>
       <c r="J3" s="9" t="inlineStr"/>
       <c r="K3" s="9" t="inlineStr"/>
     </row>
-    <row r="4" ht="92" customHeight="1">
+    <row r="4" ht="165" customHeight="1">
       <c r="A4" s="3" t="n">
         <v>18</v>
       </c>
@@ -1560,14 +1611,17 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Ya preguntáis el tipo de reforma, pero después el cliente tiene que describir el resto en texto libre. Ahí puede caber desde cambiar un baño hasta una integral de 120 m². Cada solicitud todavía requiere trabajo antes de saber si merece la pena. Os he montado una demo de cómo recoger todo eso antes de que llegue el lead: https://presupuestos.nico-soto.es/demo/grupo-g-reformas</t>
+          <t>Hola, equipo de Grupo G Reformas:
+Ya preguntáis el tipo de reforma, pero después el cliente tiene que describir el resto en texto libre. Ahí puede caber desde cambiar un baño hasta una integral de 120 m². Cada solicitud todavía requiere trabajo antes de saber si merece la pena. Os he montado una demo de cómo recoger todo eso antes de que llegue el lead:
+https://presupuestos.nico-soto.es/demo/grupo-g-reformas
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr"/>
       <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr"/>
     </row>
-    <row r="5" ht="92" customHeight="1">
+    <row r="5" ht="165" customHeight="1">
       <c r="A5" s="8" t="n">
         <v>19</v>
       </c>
@@ -1601,14 +1655,17 @@
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>He visto que vuestra solicitud recoge nombre, teléfono, email y “¿en qué podemos ayudarte?”. Es decir, prácticamente todo el trabajo de entender la reforma empieza después de recibir el lead. He montado una demo con vuestra marca para que cada solicitud os llegue con el proyecto mucho más claro antes de dedicarle tiempo: https://presupuestos.nico-soto.es/demo/azahar-reformas</t>
+          <t>Hola, equipo de Azahar Reformas Valencia:
+He visto que vuestra solicitud recoge nombre, teléfono, email y “¿en qué podemos ayudarte?”. Es decir, prácticamente todo el trabajo de entender la reforma empieza después de recibir el lead. He montado una demo con vuestra marca para que cada solicitud os llegue con el proyecto mucho más claro antes de dedicarle tiempo:
+https://presupuestos.nico-soto.es/demo/azahar-reformas
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr"/>
       <c r="J5" s="9" t="inlineStr"/>
       <c r="K5" s="9" t="inlineStr"/>
     </row>
-    <row r="6" ht="92" customHeight="1">
+    <row r="6" ht="165" customHeight="1">
       <c r="A6" s="3" t="n">
         <v>20</v>
       </c>
@@ -1642,14 +1699,17 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Me llamó la atención que os posicionéis para búsquedas de presupuesto de reforma de piso en Valencia, pero cuando llega el cliente el formulario apenas recoge sus datos y un mensaje. Cada solicitud todavía os obliga a reconstruir el proyecto antes de saber si merece la pena. He preparado una demo de cómo podría funcionar ese paso: https://presupuestos.nico-soto.es/demo/todo-reformas-valencia</t>
+          <t>Hola, equipo de Todo Reformas Valencia:
+Me llamó la atención que os posicionéis para búsquedas de presupuesto de reforma de piso en Valencia, pero cuando llega el cliente el formulario apenas recoge sus datos y un mensaje. Cada solicitud todavía os obliga a reconstruir el proyecto antes de saber si merece la pena. He preparado una demo de cómo podría funcionar ese paso:
+https://presupuestos.nico-soto.es/demo/todo-reformas-valencia
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr"/>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="4" t="inlineStr"/>
     </row>
-    <row r="7" ht="92" customHeight="1">
+    <row r="7" ht="165" customHeight="1">
       <c r="A7" s="8" t="n">
         <v>21</v>
       </c>
@@ -1683,14 +1743,17 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>Hacéis reformas integrales, cocinas y baños, pero el cliente tiene que explicar lo que quiere prácticamente desde cero en un mensaje. Luego sois vosotros quienes convertís eso en metros, estancias, trabajos e inversión. He montado una demo para enseñaros cómo podría llegaros esa información ya estructurada: https://presupuestos.nico-soto.es/demo/reformas-orcu</t>
+          <t>Hola, equipo de Reformas Orcu:
+Hacéis reformas integrales, cocinas y baños, pero el cliente tiene que explicar lo que quiere prácticamente desde cero en un mensaje. Luego sois vosotros quienes convertís eso en metros, estancias, trabajos e inversión. He montado una demo para enseñaros cómo podría llegaros esa información ya estructurada:
+https://presupuestos.nico-soto.es/demo/reformas-orcu
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr"/>
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="9" t="inlineStr"/>
     </row>
-    <row r="8" ht="92" customHeight="1">
+    <row r="8" ht="165" customHeight="1">
       <c r="A8" s="3" t="n">
         <v>22</v>
       </c>
@@ -1724,14 +1787,17 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>He visto que vuestro formulario ya pregunta cuándo quiere realizar el trabajo, pero no recoge metros, estancias, alcance ni inversión. Sabéis cuándo quiere empezar, pero todavía tenéis que averiguar casi todo lo demás antes de saber si merece la pena. He preparado una demo para completar justo esa parte: https://presupuestos.nico-soto.es/demo/obras-vip</t>
+          <t>Hola, equipo de OBRAS VIP:
+He visto que vuestro formulario ya pregunta cuándo quiere realizar el trabajo, pero no recoge metros, estancias, alcance ni inversión. Sabéis cuándo quiere empezar, pero todavía tenéis que averiguar casi todo lo demás antes de saber si merece la pena. He preparado una demo para completar justo esa parte:
+https://presupuestos.nico-soto.es/demo/obras-vip
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="4" t="inlineStr"/>
     </row>
-    <row r="9" ht="92" customHeight="1">
+    <row r="9" ht="165" customHeight="1">
       <c r="A9" s="8" t="n">
         <v>23</v>
       </c>
@@ -1765,14 +1831,17 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>Vendéis proyectos llave en mano, pero cuando alguien pide información entra por un formulario genérico y todavía tenéis que averiguar todo el alcance del proyecto. Cada solicitud os obliga a trabajar antes de saber si encaja realmente. He preparado una demo para enseñaros cómo podría llegaros mucho más definida: https://presupuestos.nico-soto.es/demo/bono-proyectos</t>
+          <t>Hola, equipo de BONO PROYECTOS:
+Vendéis proyectos llave en mano, pero cuando alguien pide información entra por un formulario genérico y todavía tenéis que averiguar todo el alcance del proyecto. Cada solicitud os obliga a trabajar antes de saber si encaja realmente. He preparado una demo para enseñaros cómo podría llegaros mucho más definida:
+https://presupuestos.nico-soto.es/demo/bono-proyectos
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr"/>
       <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="9" t="inlineStr"/>
     </row>
-    <row r="10" ht="92" customHeight="1">
+    <row r="10" ht="165" customHeight="1">
       <c r="A10" s="3" t="n">
         <v>24</v>
       </c>
@@ -1806,14 +1875,17 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>He visto que ya preguntáis el tipo de servicio, pero la cualificación se queda ahí: no metros, estancias, timing, fotos ni inversión prevista. Cada solicitud todavía os obliga a completar todo eso después. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado: https://presupuestos.nico-soto.es/demo/vga-reformas</t>
+          <t>Hola, equipo de VGA Proyectos y Reformas:
+He visto que ya preguntáis el tipo de servicio, pero la cualificación se queda ahí: no metros, estancias, timing, fotos ni inversión prevista. Cada solicitud todavía os obliga a completar todo eso después. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado:
+https://presupuestos.nico-soto.es/demo/vga-reformas
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="4" t="inlineStr"/>
     </row>
-    <row r="11" ht="92" customHeight="1">
+    <row r="11" ht="165" customHeight="1">
       <c r="A11" s="8" t="n">
         <v>25</v>
       </c>
@@ -1843,14 +1915,17 @@
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>Tenéis una página específica para solicitar presupuesto, pero al final el cliente deja sus datos y os cuenta libremente lo que necesita. El trabajo de convertir eso en un proyecto presupuestable sigue siendo vuestro. He preparado una demo para que veáis cómo podría llegaros ya estructurado antes de dedicarle tiempo: https://presupuestos.nico-soto.es/demo/reformspeed</t>
+          <t>Hola, equipo de REFORMSPEED:
+Tenéis una página específica para solicitar presupuesto, pero al final el cliente deja sus datos y os cuenta libremente lo que necesita. El trabajo de convertir eso en un proyecto presupuestable sigue siendo vuestro. He preparado una demo para que veáis cómo podría llegaros ya estructurado antes de dedicarle tiempo:
+https://presupuestos.nico-soto.es/demo/reformspeed
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr"/>
       <c r="J11" s="9" t="inlineStr"/>
       <c r="K11" s="9" t="inlineStr"/>
     </row>
-    <row r="12" ht="92" customHeight="1">
+    <row r="12" ht="165" customHeight="1">
       <c r="A12" s="3" t="n">
         <v>26</v>
       </c>
@@ -1884,14 +1959,17 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>He visto que la petición de presupuesto os llega básicamente como datos de contacto y un mensaje. Eso significa que cada nuevo lead todavía necesita una conversación para saber qué quiere, cuánto, cuándo y si realmente merece la pena presupuestarlo. He montado una demo para enseñaros cómo podría llegaros esa reforma ya explicada: https://presupuestos.nico-soto.es/demo/grupo-expovall</t>
+          <t>Hola, equipo de Valltro:
+He visto que la petición de presupuesto os llega básicamente como datos de contacto y un mensaje. Eso significa que cada nuevo lead todavía necesita una conversación para saber qué quiere, cuánto, cuándo y si realmente merece la pena presupuestarlo. He montado una demo para enseñaros cómo podría llegaros esa reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/grupo-expovall
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr"/>
     </row>
-    <row r="13" ht="92" customHeight="1">
+    <row r="13" ht="165" customHeight="1">
       <c r="A13" s="8" t="n">
         <v>27</v>
       </c>
@@ -1925,14 +2003,17 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Trabajáis cocinas, baños y reformas de pisos, pero la solicitud online no diferencia entre ninguno de esos proyectos. Cada lead os llega sin la información que determina el trabajo y sois vosotros quienes tenéis que sacársela después. He preparado una demo con vuestra marca para enseñaros otra forma de recibirlos: https://presupuestos.nico-soto.es/demo/cecever</t>
+          <t>Hola, equipo de Reformas Cecever:
+Trabajáis cocinas, baños y reformas de pisos, pero la solicitud online no diferencia entre ninguno de esos proyectos. Cada lead os llega sin la información que determina el trabajo y sois vosotros quienes tenéis que sacársela después. He preparado una demo con vuestra marca para enseñaros otra forma de recibirlos:
+https://presupuestos.nico-soto.es/demo/cecever
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr"/>
       <c r="J13" s="9" t="inlineStr"/>
       <c r="K13" s="9" t="inlineStr"/>
     </row>
-    <row r="14" ht="92" customHeight="1">
+    <row r="14" ht="165" customHeight="1">
       <c r="A14" s="3" t="n">
         <v>28</v>
       </c>
@@ -1966,14 +2047,17 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>He visto que cuando alguien contacta os deja nombre, teléfono, email y un mensaje. Es decir, todo lo importante sobre la reforma empieza después. Cada solicitud todavía os obliga a trabajar antes de saber si merece la pena. He montado una demo para enseñaros cómo podría llegaros ya cualificada: https://presupuestos.nico-soto.es/demo/reformas-ferreira</t>
+          <t>Hola, equipo de Reformas Ferreira:
+He visto que cuando alguien contacta os deja nombre, teléfono, email y un mensaje. Es decir, todo lo importante sobre la reforma empieza después. Cada solicitud todavía os obliga a trabajar antes de saber si merece la pena. He montado una demo para enseñaros cómo podría llegaros ya cualificada:
+https://presupuestos.nico-soto.es/demo/reformas-ferreira
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr"/>
     </row>
-    <row r="15" ht="92" customHeight="1">
+    <row r="15" ht="165" customHeight="1">
       <c r="A15" s="8" t="n">
         <v>29</v>
       </c>
@@ -2007,14 +2091,17 @@
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Tenéis un CTA de “Solicita presupuesto Online”, pero el proceso termina en un formulario de cuatro campos. Online es la solicitud; el trabajo de entender y presupuestar la reforma sigue viniendo después. He preparado una demo para enseñaros cómo convertir ese “presupuesto online” en algo bastante más útil: https://presupuestos.nico-soto.es/demo/dekorinex</t>
+          <t>Hola, equipo de Dekorinex:
+Tenéis un CTA de “Solicita presupuesto Online”, pero el proceso termina en un formulario de cuatro campos. Online es la solicitud; el trabajo de entender y presupuestar la reforma sigue viniendo después. He preparado una demo para enseñaros cómo convertir ese “presupuesto online” en algo bastante más útil:
+https://presupuestos.nico-soto.es/demo/dekorinex
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr"/>
       <c r="J15" s="9" t="inlineStr"/>
       <c r="K15" s="9" t="inlineStr"/>
     </row>
-    <row r="16" ht="92" customHeight="1">
+    <row r="16" ht="165" customHeight="1">
       <c r="A16" s="3" t="n">
         <v>30</v>
       </c>
@@ -2048,7 +2135,10 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Lleváis años haciendo reformas integrales, cocinas y baños, pero el formulario todavía deja prácticamente todo el proyecto dentro de un mensaje libre. Cada solicitud os obliga a interpretarla y cualificarla antes de saber si merece la pena. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada reforma ya explicada: https://presupuestos.nico-soto.es/demo/incoval</t>
+          <t>Hola, equipo de Incoval Reformas Integrales:
+Lleváis años haciendo reformas integrales, cocinas y baños, pero el formulario todavía deja prácticamente todo el proyecto dentro de un mensaje libre. Cada solicitud os obliga a interpretarla y cualificarla antes de saber si merece la pena. He montado una demo con vuestra marca para que veáis cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/incoval
+Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
docs(prospeccion): resultado del lote 1 y avisos del lote 2 en la cola de envío
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -8,12 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Leeme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Hoy (1-15)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Manana (16-30)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lote 1 (1-15) enviado" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lote 2 (16-30)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hoy (1-15)'!$A$1:$K$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Manana (16-30)'!$A$1:$K$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lote 1 (1-15) enviado'!$A$1:$L$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lote 2 (16-30)'!$A$1:$L$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <name val="Calibri"/>
@@ -106,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -144,6 +147,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -510,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -523,26 +535,22 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hoja 'Hoy (1-15)': leads 1 a 15 de la auditoria (scores 9,5 - 7,5).</t>
+          <t>Hoja 'Lote 1 (1-15) enviado': enviados el 25/08/2026 por formulario web. Resultado a 12/09: 7 de 15 abrieron la demo, 1 interesado real (ROBLES Home), 0 respuestas.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hoja 'Manana (16-30)': leads 16 a 30 (scores 7,5 - 7,0).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+          <t>Hoja 'Lote 2 (16-30)': 15 pendientes, demos y formularios verificados el 12/09. Marca Enviado = Sí y la fecha al enviar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -560,13 +568,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>con su logo y sus colores. Verificado: las 30 responden 200.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+          <t>con su logo y sus colores. Verificado el 12/09: las 15 del lote 2 responden 200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
@@ -588,13 +594,25 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
           <t>Lead 25 (REFORMSPEED) no tiene email: solo contacto por formulario web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Lead 23 (BONO PROYECTOS): el email tiene errata, usar el formulario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>'Demo abierta' sale de la analítica del proyecto Lovable reform-wizard (visitas 25/08-12/09; pueden incluir pruebas propias).</t>
         </is>
       </c>
     </row>
@@ -609,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -622,7 +640,8 @@
     <col width="95" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -681,6 +700,11 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Demo abierta</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="165" customHeight="1">
       <c r="A2" s="3" t="n">
@@ -722,9 +746,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>Abrió la demo, no dejó datos. OJO: también tiene web construida en WebForge; elegir un producto antes de insistir.</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>Sí · 2 visitas</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="165" customHeight="1">
       <c r="A3" s="8" t="n">
@@ -766,9 +805,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr"/>
-      <c r="J3" s="9" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr"/>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J3" s="16" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>Abrió la demo, no dejó datos.</t>
+        </is>
+      </c>
+      <c r="L3" s="15" t="inlineStr">
+        <is>
+          <t>Sí · 1 visita</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="165" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -810,9 +864,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr"/>
-      <c r="J4" s="4" t="inlineStr"/>
-      <c r="K4" s="4" t="inlineStr"/>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Abrió la demo, no dejó datos.</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>Sí · 3 visitas</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="165" customHeight="1">
       <c r="A5" s="8" t="n">
@@ -854,9 +923,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I5" s="9" t="inlineStr"/>
-      <c r="J5" s="9" t="inlineStr"/>
-      <c r="K5" s="9" t="inlineStr"/>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Nunca abrió la demo.</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="165" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -898,9 +982,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Nunca abrió la demo.</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="165" customHeight="1">
       <c r="A7" s="8" t="n">
@@ -942,9 +1041,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="9" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>Nunca abrió la demo.</t>
+        </is>
+      </c>
+      <c r="L7" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="165" customHeight="1">
       <c r="A8" s="3" t="n">
@@ -986,9 +1100,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
-      <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>El "lead" del 26/08 era una prueba propia (tel 600782211), no el cliente. Sin respuesta real.</t>
+        </is>
+      </c>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>Sí · 4 visitas</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="165" customHeight="1">
       <c r="A9" s="8" t="n">
@@ -1030,9 +1159,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr"/>
-      <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>Nunca abrió la demo. Contactan por WhatsApp/teléfono.</t>
+        </is>
+      </c>
+      <c r="L9" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="165" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1074,9 +1218,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>ÚNICO INTERESADO REAL: completó el wizard el 25/08 13:15 (casa 65 m², 46900, integral+ventanas+puertas+clima, 50-100K; horquilla 40.010-74.300 €). Tel 605459217 ≈ oficial 605459216. Seguimiento por email enviado 12/09 a info@robleshome.com.</t>
+        </is>
+      </c>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>Sí · 5 visitas</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="165" customHeight="1">
       <c r="A11" s="8" t="n">
@@ -1118,9 +1277,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>Abrió la demo, no dejó datos.</t>
+        </is>
+      </c>
+      <c r="L11" s="15" t="inlineStr">
+        <is>
+          <t>Sí · 1 visita</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="165" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1162,9 +1336,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="4" t="inlineStr"/>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>Nunca abrió la demo.</t>
+        </is>
+      </c>
+      <c r="L12" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="165" customHeight="1">
       <c r="A13" s="8" t="n">
@@ -1206,9 +1395,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I13" s="9" t="inlineStr"/>
-      <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>Nunca abrió la demo.</t>
+        </is>
+      </c>
+      <c r="L13" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="165" customHeight="1">
       <c r="A14" s="3" t="n">
@@ -1250,9 +1454,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" s="4" t="inlineStr"/>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>Abrió la demo, no dejó datos.</t>
+        </is>
+      </c>
+      <c r="L14" s="15" t="inlineStr">
+        <is>
+          <t>Sí · 2 visitas</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="165" customHeight="1">
       <c r="A15" s="8" t="n">
@@ -1294,9 +1513,24 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I15" s="9" t="inlineStr"/>
-      <c r="J15" s="9" t="inlineStr"/>
-      <c r="K15" s="9" t="inlineStr"/>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>Nunca abrió la demo.</t>
+        </is>
+      </c>
+      <c r="L15" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="165" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -1338,12 +1572,27 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>46259</v>
+      </c>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>Nunca abrió la demo.</t>
+        </is>
+      </c>
+      <c r="L16" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K16"/>
+  <autoFilter ref="A1:L16"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -1416,7 +1665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1429,7 +1678,8 @@
     <col width="95" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1488,6 +1738,11 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Demo abierta</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="165" customHeight="1">
       <c r="A2" s="3" t="n">
@@ -1529,9 +1784,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr"/>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200).</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="165" customHeight="1">
       <c r="A3" s="8" t="n">
@@ -1573,9 +1836,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr"/>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J3" s="9" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr"/>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200).</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="165" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1617,9 +1888,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr"/>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J4" s="4" t="inlineStr"/>
-      <c r="K4" s="4" t="inlineStr"/>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200). Sin página de contacto: el formulario está en la home.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="165" customHeight="1">
       <c r="A5" s="8" t="n">
@@ -1661,9 +1940,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I5" s="9" t="inlineStr"/>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J5" s="9" t="inlineStr"/>
-      <c r="K5" s="9" t="inlineStr"/>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200).</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="165" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1705,9 +1992,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr"/>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200).</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="165" customHeight="1">
       <c r="A7" s="8" t="n">
@@ -1749,9 +2044,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J7" s="9" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200).</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="165" customHeight="1">
       <c r="A8" s="3" t="n">
@@ -1793,9 +2096,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200). Su demo lleva el nombre en su color (logo de la web solo a 50 px).</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="165" customHeight="1">
       <c r="A9" s="8" t="n">
@@ -1837,9 +2148,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr"/>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200). OJO email con errata: info@bonoporyectos.com (web es bonoproyectos.es). Usar el formulario, no ese email.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="165" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1881,9 +2200,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200). Sin página de contacto: la home lleva dos formularios duplicados, usa uno.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="165" customHeight="1">
       <c r="A11" s="8" t="n">
@@ -1921,9 +2248,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr"/>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>Demo verificada 12/09 (200). Sin email. Su página /solicitar-presupuesto/ daba error 500 el 12/09: comprobar antes de enviar.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="165" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1965,9 +2300,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="4" t="inlineStr"/>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200).</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="165" customHeight="1">
       <c r="A13" s="8" t="n">
@@ -2009,9 +2352,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I13" s="9" t="inlineStr"/>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200).</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="165" customHeight="1">
       <c r="A14" s="3" t="n">
@@ -2053,9 +2404,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr"/>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" s="4" t="inlineStr"/>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200). Sin página de contacto: localiza el formulario en la home.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="165" customHeight="1">
       <c r="A15" s="8" t="n">
@@ -2097,9 +2456,17 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I15" s="9" t="inlineStr"/>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J15" s="9" t="inlineStr"/>
-      <c r="K15" s="9" t="inlineStr"/>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200).</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="165" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2141,12 +2508,20 @@
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr"/>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>Demo y formulario verificados 12/09 (200).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K16"/>
+  <autoFilter ref="A1:L16"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>

</xml_diff>

<commit_message>
docs(prospeccion): REFORMSPEED (#25) pasa a WhatsApp manual, su web da 500
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -21,9 +21,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -109,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -148,13 +147,19 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -535,7 +540,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -550,7 +554,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -572,7 +575,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
@@ -594,11 +596,10 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Lead 25 (REFORMSPEED) no tiene email: solo contacto por formulario web.</t>
+          <t>Lead 25 (REFORMSPEED) no tiene email y su web da error 500: se contacta por WhatsApp manual al +34 631 02 90 72 (Google Maps)</t>
         </is>
       </c>
     </row>
@@ -751,7 +752,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J2" s="14" t="n">
+      <c r="J2" s="17" t="n">
         <v>46259</v>
       </c>
       <c r="K2" s="7" t="inlineStr">
@@ -810,7 +811,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J3" s="16" t="n">
+      <c r="J3" s="18" t="n">
         <v>46259</v>
       </c>
       <c r="K3" s="11" t="inlineStr">
@@ -869,7 +870,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="17" t="n">
         <v>46259</v>
       </c>
       <c r="K4" s="7" t="inlineStr">
@@ -928,7 +929,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J5" s="16" t="n">
+      <c r="J5" s="18" t="n">
         <v>46259</v>
       </c>
       <c r="K5" s="11" t="inlineStr">
@@ -987,7 +988,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="17" t="n">
         <v>46259</v>
       </c>
       <c r="K6" s="7" t="inlineStr">
@@ -1046,7 +1047,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J7" s="16" t="n">
+      <c r="J7" s="18" t="n">
         <v>46259</v>
       </c>
       <c r="K7" s="11" t="inlineStr">
@@ -1105,7 +1106,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J8" s="14" t="n">
+      <c r="J8" s="17" t="n">
         <v>46259</v>
       </c>
       <c r="K8" s="7" t="inlineStr">
@@ -1164,7 +1165,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J9" s="16" t="n">
+      <c r="J9" s="18" t="n">
         <v>46259</v>
       </c>
       <c r="K9" s="11" t="inlineStr">
@@ -1223,7 +1224,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="17" t="n">
         <v>46259</v>
       </c>
       <c r="K10" s="7" t="inlineStr">
@@ -1282,7 +1283,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J11" s="16" t="n">
+      <c r="J11" s="18" t="n">
         <v>46259</v>
       </c>
       <c r="K11" s="11" t="inlineStr">
@@ -1341,7 +1342,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J12" s="14" t="n">
+      <c r="J12" s="17" t="n">
         <v>46259</v>
       </c>
       <c r="K12" s="7" t="inlineStr">
@@ -1400,7 +1401,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J13" s="16" t="n">
+      <c r="J13" s="18" t="n">
         <v>46259</v>
       </c>
       <c r="K13" s="11" t="inlineStr">
@@ -1459,7 +1460,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J14" s="14" t="n">
+      <c r="J14" s="17" t="n">
         <v>46259</v>
       </c>
       <c r="K14" s="7" t="inlineStr">
@@ -1518,7 +1519,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J15" s="16" t="n">
+      <c r="J15" s="18" t="n">
         <v>46259</v>
       </c>
       <c r="K15" s="11" t="inlineStr">
@@ -1577,7 +1578,7 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="17" t="n">
         <v>46259</v>
       </c>
       <c r="K16" s="7" t="inlineStr">
@@ -2227,7 +2228,7 @@
       <c r="D11" s="9" t="inlineStr"/>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>https://reformspeed.es/solicitar-presupuesto/</t>
+          <t>https://wa.me/34631029072</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
@@ -2256,7 +2257,7 @@
       <c r="J11" s="9" t="inlineStr"/>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>Demo verificada 12/09 (200). Sin email. Su página /solicitar-presupuesto/ daba error 500 el 12/09: comprobar antes de enviar.</t>
+          <t>Por WhatsApp (+34 631 02 90 72, móvil de Google Maps): su web entera da error 500 el 12 y 13/09 y no tiene email. Mismo mensaje, envío manual.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(prospeccion): lote 3 del simulador en la cola, con sus 15 demos de marca
Quince empresas más (31-45) debajo del lote 2: logo y color sacados del logo
de cada web, mensaje por empresa con su ángulo de la auditoría, CSV y hoja
nueva en el Excel.

Aquí tu Reforma se cae al revisar (cadena nacional con franquicias y su propio
formulario de 7 pasos); entra Reformas Génesis, primera reserva. Estil Nou
Miravet va por WhatsApp porque no tiene formulario. Los logos blancos de
Renovat y Estil Nou llevan versión sobre fondo oscuro (-fondo.png) para la
demo de presupuestos.nico-soto.es, que los pinta sobre fondo claro.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -10,10 +10,12 @@
     <sheet name="Leeme" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Lote 1 (1-15) enviado" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Lote 2 (16-30)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lote 3 (31-45)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lote 1 (1-15) enviado'!$A$1:$L$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lote 2 (16-30)'!$A$1:$L$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lote 3 (31-45)'!$A$1:$L$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -527,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -540,6 +542,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -554,66 +557,84 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hoja 'Lote 3 (31-45)': 15 pendientes, montado el 13/09 (auditoría Safor y Ribera + fichas A de agosto). Aquí tu Reforma descartada al revisar; entra Reformas Génesis (reserva 16).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Enlace de la demo</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Cada lead tiene su preview de marca en https://presupuestos.nico-soto.es/demo/&lt;slug&gt;,</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Cada lead tiene su preview de marca en https://presupuestos.nico-soto.es/demo/&lt;slug&gt;,</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>con su logo y sus colores. Verificado el 12/09: las 15 del lote 2 responden 200.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Datos para rellenar los formularios</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Email de respuesta:  hola@nico-soto.es</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Email de respuesta:  hola@nico-soto.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Telefono / WhatsApp: +34 600 78 22 11</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Lead 25 (REFORMSPEED) no tiene email y su web da error 500: se contacta por WhatsApp manual al +34 631 02 90 72 (Google Maps)</t>
-        </is>
-      </c>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lead 23 (BONO PROYECTOS): el email tiene errata, usar el formulario.</t>
+          <t>Lead 25 (REFORMSPEED) no tiene email y su web da error 500: se contacta por WhatsApp manual al +34 631 02 90 72 (Google Maps)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Lead 23 (BONO PROYECTOS): el email tiene errata, usar el formulario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>'Demo abierta' sale de la analítica del proyecto Lovable reform-wizard (visitas 25/08-12/09; pueden incluir pruebas propias).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Lead 37 (Estil Nou Miravet) no tiene formulario ni email: WhatsApp manual al +34 650 40 88 34.</t>
         </is>
       </c>
     </row>
@@ -2586,4 +2607,988 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>URL contacto</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Demo (URL)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje (listo para enviar)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha envio</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Demo abierta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="165" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Renovat Reformas</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>info@reformasrenovat.com</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>https://www.reformasrenovat.com/</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>http://www.reformasrenovat.com</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/renovat-reformas</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Renovat Reformas:
+He visto vuestro bloque de "Pide presupuesto sin compromiso": seis campos obligatorios (nombre, apellidos, email, teléfono, asunto y mensaje) y ninguno pregunta por la reforma. Con casi 150 reseñas, cada solicitud que entra todavía os obliga a averiguar metros, estancias e inversión antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros ya explicada:
+https://presupuestos.nico-soto.es/demo/renovat-reformas
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="n"/>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). El formulario está en la home, en el bloque «Pide presupuesto sin compromiso» (no hay página de contacto aparte).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="165" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Reformas y Pintores Nico</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>pintoresnico@gmail.com</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>https://xn--reformaypintoresnicoespaa-woc.com/es</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>https://xn--reformaypintoresnicoespaa-woc.com</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-pintores-nico</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas y Pintores Nico:
+Con más de 500 reseñas, imagino que os entra de todo. Por el mismo formulario de nombre, email, teléfono y mensaje os llega igual pintar un salón que una reforma integral, y no lo sabéis hasta que llamáis. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada solicitud ya separada y explicada:
+https://presupuestos.nico-soto.es/demo/reformas-pintores-nico
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="n"/>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). El formulario está en la home y lleva reCAPTCHA. Mezcla reformas con pintura y comunidades: si se trata como B, su score baja a ~7,5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="165" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Mestre Reformas</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>info@mestrereformas.com</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.mestrereformas.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.mestrereformas.com</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/mestre-reformas</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Mestre Reformas:
+Prometéis precios cerrados y presupuesto en menos de 48 horas, pero el formulario de contacto solo pide nombre, correo y mensaje: ni teléfono, ni metros, ni qué estancia. Para cumplir esas 48 horas, lo primero es perseguir al cliente para saber qué quiere. He montado una demo con vuestra marca para enseñaros cómo podría llegaros la reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/mestre-reformas
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). Su botón «Solicita tu presupuesto Gratis» de la home es solo un enlace de teléfono: el formulario está en /contacto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="165" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Reformas Villa</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>https://www.reformasvilla.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>http://www.reformasvilla.com</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-villa</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas Villa:
+Vuestros proyectos son pisos completos, reformas integrales, cocinas y baños, pero por la web solo os llega un nombre, un email y un mensaje. Cada solicitud os obliga a empezar preguntando lo básico antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma con metros, estancias, plazo e inversión ya recogidos:
+https://presupuestos.nico-soto.es/demo/reformas-villa
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="n"/>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="165" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Macamon Reformas Integrales</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>macamoncho@gmail.com</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>https://macamoncho.es/presupuestos/</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>http://macamoncho.es</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/macamon-reformas</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Macamon Reformas:
+Vuestra página "Pide tu presupuesto a medida" ya pregunta qué necesita el cliente y para dónde, que es más de lo que hace casi todo el sector. Pero lo recoge en texto libre: ni metros, ni plazo, ni con cuánto cuenta. He preparado una demo con vuestra marca para completar justo esa parte:
+https://presupuestos.nico-soto.es/demo/macamon-reformas
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). Lleva reCAPTCHA v3 (invisible): no debería pedirte nada, pero si el envío falla, prueba desde otro navegador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="165" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Hidro2 Grup</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>info@hidro2grup.com</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>https://www.hidro2grup.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>https://www.hidro2grup.com</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/hidro2-grup</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Hidro2 Grup:
+En vuestra web un cliente cuenta que fuisteis a medir en 48 horas y tuvo el presupuesto detallado en una semana. Es muy buen servicio, pero el formulario (nombre, email, teléfono y mensaje) no adelanta nada de esa semana: todo empieza cuando ya ha llegado el lead. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado antes de desplazaros:
+https://presupuestos.nico-soto.es/demo/hidro2-grup
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="165" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Estil Nou Miravet</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>https://wa.me/34650408834</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>https://estilnoumiravet.com</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/estil-nou-miravet</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Estil Nou Miravet:
+He visto que vuestro botón "Solicitar presupuesto" abre directamente un WhatsApp. Eso hace que cada reforma empiece con una conversación desde cero: qué quiere hacer, metros, estancias, plazo e inversión, antes de saber siquiera si merece la pena. He montado una demo con vuestra marca para que todo eso os llegue recogido antes de empezar a hablar:
+https://presupuestos.nico-soto.es/demo/estil-nou-miravet
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Por WhatsApp (sin formulario). Por WhatsApp, no por formulario: no tiene formulario ni email; todos los «Solicitar presupuesto» de su web abren WhatsApp. El enlace abre WhatsApp con su móvil (+34 650 40 88 34). Pega el mismo mensaje, a mano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="165" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Reformas Antoine</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>nikolaytsverkov@gmail.com</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>https://reformasytrasterosantuine.com/es</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>https://reformasytrasterosantuine.com</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-antoine</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas Antoine:
+Hacéis desde pequeñas reparaciones hasta reformas completas, y las dos os llegan por el mismo formulario de nombre, email, teléfono y mensaje. Hasta que no habláis con el cliente no sabéis si es un arreglo de una tarde o una obra de dos meses. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada solicitud ya explicada:
+https://presupuestos.nico-soto.es/demo/reformas-antoine
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="n"/>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). Clase B: además de reformas alquila trasteros. El formulario está en la home y lleva reCAPTCHA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="165" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Reformas integrales Cuinex</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>info@cuinexreformas.es</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>https://www.cuinexreformas.es/contacto</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>http://www.cuinexreformas.es</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/cuinex</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Cuinex:
+Me llamó la atención que vuestro formulario pida el DNI o NIF del cliente, pero no qué quiere reformar ni cuántos metros tiene. Sabéis quién es antes de saber si el proyecto merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/cuinex
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). Clase B: tira mucho a cocinas y carpintería. El formulario pregunta si eres particular o empresa y pide DNI/NIF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="165" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Jesbal Habitatge</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>info@jesbalhabitatge.es</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>https://jesbalhabitatge.es/contacto/</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>https://jesbalhabitatge.es</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/jesbal-habitatge</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Jesbal Habitatge:
+Vuestra web ya explica que una integral de unos 100 m² lleva 2-3 meses y que ayudáis con la financiación, pero el formulario solo pregunta el tipo de reforma: ni metros, ni plazo, ni inversión. Justo lo que sabéis explicar tan bien es lo que no llega en la solicitud. He montado una demo con vuestra marca para enseñaros cómo podría llegaros ya completa:
+https://presupuestos.nico-soto.es/demo/jesbal-habitatge
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="165" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Gytech group</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>info@gytechgroup.com</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>https://gytechgroup.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>https://gytechgroup.com</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/gytech-group</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Gytech:
+Ofrecéis presupuesto sin compromiso, pero hasta saber si el proyecto es real el compromiso lo ponéis vosotros: llamadas, desplazamiento, medición y horas de presupuesto. Y el formulario solo recoge nombre, email, teléfono, asunto y mensaje. He montado una demo con vuestra marca para enseñaros cómo entender el proyecto antes de dedicarle ese tiempo:
+https://presupuestos.nico-soto.es/demo/gytech-group
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="165" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Construcciones y Reformas Génesis</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>contacto@reformasgenesis.com.es</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>https://www.reformasgenesis.com.es/</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>http://www.reformasgenesis.com.es</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-genesis</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas Génesis:
+Hacéis de todo, desde un baño o una cocina hasta una reforma integral, una piscina o una nave, y por la web os llega igual: nombre, email y un mensaje. Hasta que no habláis con el cliente no sabéis cuál de todas es ni si merece la pena el desplazamiento. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/reformas-genesis
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="n"/>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). Entra por Aquí tu Reforma, que se cae: es una cadena nacional con tiendas y franquicias y ya tiene su propio formulario de presupuesto de 7 pasos. El formulario está en la home, al final (nombre, email, mensaje). También tiene WhatsApp (+34 613 36 88 72) por si falla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="165" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Reformas y Proyectos Sacaber</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>sacaber@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>http://sacaber.com/contacto</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>http://sacaber.com</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/sacaber</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas Sacaber:
+He visto que vuestro formulario recoge nombre, email, teléfono y un mensaje, y poco más. Es decir, todo el trabajo de entender la reforma (metros, estancias, alcance, inversión) empieza cuando ya ha llegado el lead. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado:
+https://presupuestos.nico-soto.es/demo/sacaber
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="165" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Construcciones y Reformas Ramírez Castañeda</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>ramirezcastanedasl@gmail.com</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>https://www.xn--construccionesyreformasramirezcastaedasl-n2d.es/contactanos</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>http://xn--construccionesyreformasramirezcastaedasl-n2d.es</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/ramirez-castaneda</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Construcciones y Reformas Ramírez Castañeda:
+He visto que en vuestra página de contacto el cliente os deja sus datos y un mensaje libre. Todo lo que determina el presupuesto (qué quiere reformar, metros, plazo e inversión) tenéis que sacarlo después, llamada a llamada. He preparado una demo con vuestra marca para enseñaros cómo podría llegaros ya recogido:
+https://presupuestos.nico-soto.es/demo/ramirez-castaneda
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="n"/>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="165" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Multiservicios AM Levante</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>multiserviciosam375@gmail.com</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>https://www.multiserviciosamlevante.es/contactanos</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>http://www.multiserviciosamlevante.es</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/multiservicios-am-levante</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Multiservicios AM Levante:
+Hacéis reformas integrales y ofrecéis presupuesto sin compromiso, pero hasta saber si el proyecto es real el compromiso lo ponéis vosotros: llamadas, visita, medición y preparar el presupuesto. Por la web solo os llegan unos datos y un mensaje. He montado una demo con vuestra marca para enseñaros cómo entender el proyecto antes de dedicarle ese tiempo:
+https://presupuestos.nico-soto.es/demo/multiservicios-am-levante
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). También tiene WhatsApp (+34 623 26 65 67), por si el formulario falla.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L16"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId59"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(prospeccion): lote 3 montado, con las demos verificadas en el Excel y el documento
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -2746,7 +2746,7 @@
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). El formulario está en la home, en el bloque «Pide presupuesto sin compromiso» (no hay página de contacto aparte).</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). El formulario está en la home, en el bloque «Pide presupuesto sin compromiso» (no hay página de contacto aparte).</t>
         </is>
       </c>
     </row>
@@ -2802,7 +2802,7 @@
       <c r="J3" s="9" t="n"/>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). El formulario está en la home y lleva reCAPTCHA. Mezcla reformas con pintura y comunidades: si se trata como B, su score baja a ~7,5.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). El formulario está en la home y lleva reCAPTCHA. Mezcla reformas con pintura y comunidades: si se trata como B, su score baja a ~7,5.</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2858,7 @@
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). Su botón «Solicita tu presupuesto Gratis» de la home es solo un enlace de teléfono: el formulario está en /contacto.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Su botón «Solicita tu presupuesto Gratis» de la home es solo un enlace de teléfono: el formulario está en /contacto.</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       <c r="J5" s="9" t="n"/>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2966,7 @@
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). Lleva reCAPTCHA v3 (invisible): no debería pedirte nada, pero si el envío falla, prueba desde otro navegador.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Lleva reCAPTCHA v3 (invisible): no debería pedirte nada, pero si el envío falla, prueba desde otro navegador.</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3022,7 @@
       <c r="J7" s="9" t="n"/>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3074,7 @@
       <c r="J8" s="4" t="n"/>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Por WhatsApp (sin formulario). Por WhatsApp, no por formulario: no tiene formulario ni email; todos los «Solicitar presupuesto» de su web abren WhatsApp. El enlace abre WhatsApp con su móvil (+34 650 40 88 34). Pega el mismo mensaje, a mano.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Por WhatsApp (sin formulario). Por WhatsApp, no por formulario: no tiene formulario ni email; todos los «Solicitar presupuesto» de su web abren WhatsApp. El enlace abre WhatsApp con su móvil (+34 650 40 88 34). Pega el mismo mensaje, a mano.</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
       <c r="J9" s="9" t="n"/>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). Clase B: además de reformas alquila trasteros. El formulario está en la home y lleva reCAPTCHA.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Clase B: además de reformas alquila trasteros. El formulario está en la home y lleva reCAPTCHA.</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3186,7 @@
       <c r="J10" s="4" t="n"/>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). Clase B: tira mucho a cocinas y carpintería. El formulario pregunta si eres particular o empresa y pide DNI/NIF.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Clase B: tira mucho a cocinas y carpintería. El formulario pregunta si eres particular o empresa y pide DNI/NIF.</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       <c r="J11" s="9" t="n"/>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
       <c r="J13" s="9" t="n"/>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). Entra por Aquí tu Reforma, que se cae: es una cadena nacional con tiendas y franquicias y ya tiene su propio formulario de presupuesto de 7 pasos. El formulario está en la home, al final (nombre, email, mensaje). También tiene WhatsApp (+34 613 36 88 72) por si falla.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Entra por Aquí tu Reforma, que se cae: es una cadena nacional con tiendas y franquicias y ya tiene su propio formulario de presupuesto de 7 pasos. El formulario está en la home, al final (nombre, email, mensaje). También tiene WhatsApp (+34 613 36 88 72) por si falla.</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3410,7 @@
       <c r="J14" s="4" t="n"/>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3466,7 @@
       <c r="J15" s="9" t="n"/>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200).</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3522,7 @@
       <c r="J16" s="4" t="n"/>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 (200). También tiene WhatsApp (+34 623 26 65 67), por si el formulario falla.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). También tiene WhatsApp (+34 623 26 65 67), por si el formulario falla.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(prospeccion): lote 4 del simulador en la cola, con sus 15 demos de marca
Lo mejor que quedaba de las auditorías (46-60, score 6,5-5,5): logo y color
sacados del logo de cada web, mensaje por empresa a partir de lo que dice su
propia web, CSV y hoja nueva en el Excel.

Al revisar en Chrome se caen Gala Projectes (almacén de materiales), Ruiz
Construcciones (contacto 404, sin formulario) y Reformas Moncada (sin
formulario); entran Proyecta Lara, Salvicar y ObraEstil.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -11,11 +11,13 @@
     <sheet name="Lote 1 (1-15) enviado" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Lote 2 (16-30)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Lote 3 (31-45)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lote 4 (46-60)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lote 1 (1-15) enviado'!$A$1:$L$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lote 2 (16-30)'!$A$1:$L$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lote 3 (31-45)'!$A$1:$L$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Lote 4 (46-60)'!$A$1:$L$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -529,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -564,75 +566,82 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Hoja 'Lote 4 (46-60)': 15 pendientes, montado el 13/09 con lo mejor que quedaba de las auditorías (score 6,5-5,5). Descartadas al revisar: Gala Projectes (almacén de materiales), Ruiz Construcciones (contacto 404, sin formulario) y Reformas Moncada (sin formulario).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Enlace de la demo</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Cada lead tiene su preview de marca en https://presupuestos.nico-soto.es/demo/&lt;slug&gt;,</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Cada lead tiene su preview de marca en https://presupuestos.nico-soto.es/demo/&lt;slug&gt;,</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>con su logo y sus colores. Verificado el 12/09: las 15 del lote 2 responden 200.</t>
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>Datos para rellenar los formularios</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Email de respuesta:  hola@nico-soto.es</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Email de respuesta:  hola@nico-soto.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Telefono / WhatsApp: +34 600 78 22 11</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Lead 25 (REFORMSPEED) no tiene email y su web da error 500: se contacta por WhatsApp manual al +34 631 02 90 72 (Google Maps)</t>
-        </is>
-      </c>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lead 23 (BONO PROYECTOS): el email tiene errata, usar el formulario.</t>
+          <t>Lead 25 (REFORMSPEED) no tiene email y su web da error 500: se contacta por WhatsApp manual al +34 631 02 90 72 (Google Maps)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Lead 23 (BONO PROYECTOS): el email tiene errata, usar el formulario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>'Demo abierta' sale de la analítica del proyecto Lovable reform-wizard (visitas 25/08-12/09; pueden incluir pruebas propias).</t>
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Lead 37 (Estil Nou Miravet) no tiene formulario ni email: WhatsApp manual al +34 650 40 88 34.</t>
         </is>
@@ -2878,7 +2887,11 @@
           <t>8.0</t>
         </is>
       </c>
-      <c r="D5" s="10" t="n"/>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>mailto:hola@azaharreformasvalencia.com</t>
+        </is>
+      </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
           <t>https://www.reformasvilla.com/contacto/</t>
@@ -3042,7 +3055,11 @@
           <t>7.5</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n"/>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>mailto:info@obrasvip.com</t>
+        </is>
+      </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
           <t>https://wa.me/34650408834</t>
@@ -3523,6 +3540,994 @@
       <c r="K16" s="7" t="inlineStr">
         <is>
           <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). También tiene WhatsApp (+34 623 26 65 67), por si el formulario falla.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L16"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId59"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>URL contacto</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Demo (URL)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje (listo para enviar)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha envio</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Demo abierta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="165" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Ecerotres Arquitectos</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>estudio@ecerotresarquitectos.com</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>https://ecerotresarquitectos.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>https://ecerotresarquitectos.com</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/ecerotres</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Ecerotres Arquitectos:
+En vuestra web explicáis bien el método: mediciones por partidas, presupuesto de obra, plan de obra y plazos. Pero antes de llegar ahí, el formulario solo os deja nombre, correo, teléfono y un mensaje, y cada solicitud empieza con una conversación para saber qué quiere reformar el cliente, cuántos metros tiene y con qué presupuesto cuenta. He montado una demo con vuestra marca para enseñaros cómo podría llegaros ese primer paso ya hecho:
+https://presupuestos.nico-soto.es/demo/ecerotres
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="n"/>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: estudio de arquitectura que hace reformas íntegras de vivienda y locales (56 reseñas, 4,9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="165" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>extraMURS Arquitectura</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>info@extramurs.com</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>https://extramurs.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>https://extramurs.com</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/extramurs</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de extraMURS:
+Vuestro blog responde cuánto cuesta construir una casa o una licencia de obra, y ofrecéis calcular una estimación de precio y plazos. Pero quien llega al formulario solo puede contaros en "¿Qué necesitas?" lo que tiene en mente, y esa estimación la preparáis vosotros después, a mano. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada, con metros, alcance, plazo e inversión:
+https://presupuestos.nico-soto.es/demo/extramurs
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="n"/>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: constructora y estudio de arquitectura, con obra nueva además de reformas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="165" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Proyecta Lara</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>comercial@proyectalara.es</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>https://proyectalara.es/</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>https://proyectalara.es</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/proyecta-lara</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Proyecta Lara:
+Prometéis reformas llave en mano con plazo y presupuesto cerrado, ajustadas a lo que puede invertir cada cliente. Pero para pediros información, en la web solo se puede dejar un email y poco más: no sabéis qué quiere reformar, cuántos metros tiene ni con cuánto cuenta hasta que habláis con él. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada proyecto ya definido:
+https://presupuestos.nico-soto.es/demo/proyecta-lara
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: estudio de interiorismo. El formulario está al pie de la home (email y un campo más) y lleva reCAPTCHA; la página «Contacta con nosotros» no tiene formulario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="165" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Construcciones OLBE</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>info@construccionesoliver.es</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>https://construccionesolbe.com/</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>https://www.construccionesolbe.com</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/construcciones-olbe</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Construcciones OLBE:
+Hacéis desde obra pequeña, una cocina o un baño, hasta reformas integrales llave en mano y trabajos en fincas, y todo os llega por el mismo formulario de nombre, email y mensaje. Hasta que no habláis con el cliente no sabéis cuál de todos es ni si merece la pena ir a verlo. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada solicitud ya explicada:
+https://presupuestos.nico-soto.es/demo/construcciones-olbe
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="n"/>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. El formulario está al final de la home (no hay página de contacto aparte). El email de su ficha es de otro dominio (construccionesoliver.es): usa el formulario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="165" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Construcciones y Reformas Clurjor</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>info@clurjor.com</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>http://clurjor.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>http://www.clurjor.com</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/clurjor</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Clurjor:
+Vuestro formulario pregunta "¿Qué necesitas?" y "Explícanos un poco más", que ya es más que muchos. Pero ahí cabe igual un baño que un local entero, y los metros, el plazo o la inversión los tenéis que sacar después, llamada a llamada. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/clurjor
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Hacen también obra nueva, locales y naves: la reforma de vivienda es una parte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="165" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>NCA Interiores</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>administracion@ncainteriores.es</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>https://ncainteriores.es/contacto/</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>https://ncainteriores.es</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/nca-interiores</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de NCA Interiores:
+Ya enseñáis la cocina en un 3D realista antes de hacerla, así que vuestro cliente entiende el valor de saber cómo quedará antes de decidir. Pero para llegar a ese punto la solicitud sigue siendo nombre, teléfono y un comentario, y las medidas, el alcance y la inversión los recogéis vosotros después. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada proyecto ya explicado:
+https://presupuestos.nico-soto.es/demo/nca-interiores
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: cocinas, armarios y carpintería a medida más que reforma integral. El formulario lleva reCAPTCHA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="165" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Obralis</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>https://obralis.es/contacto/</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>https://obralis.es</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/obralis</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Obralis:
+Vuestra web promete "Presupuesto Ahora" y un presupuesto ágil y gratis, pero el formulario pide nombre, teléfono, email y asunto, y después toca llamar y hacer la visita. El "ahora" empieza varios días más tarde. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada antes de coger el teléfono:
+https://presupuestos.nico-soto.es/demo/obralis
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. No tiene email en la ficha. También tiene WhatsApp en la web, por si el formulario falla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="165" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Mesform Interiorismo</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>info@mesform.es</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>https://www.mesform.es/contactame/</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>http://mesform.es</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/mesform</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Mesform:
+Hacéis desde muebles y vestidores a medida hasta reformas integrales, y vuestro "Contáctame" lo recibe todo igual: nombre, email y mensaje. Hasta que no habláis con el cliente no sabéis si es un armario o un piso entero. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada proyecto ya explicado:
+https://presupuestos.nico-soto.es/demo/mesform
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="n"/>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: interiorismo y carpintería a medida con reformas. El email de su ficha es de relleno (contacto@ejemplo.com); el real de su web es info@mesform.es. Usa el formulario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="165" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Tres i Tres Interiorismo</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>info@3itres.com</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>https://3itres.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>http://3itres.com</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/tres-i-tres</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Tres i Tres:
+Ponéis mucho el foco en la gestión de plazos y en garantizar las fechas de entrega, pero cada "pídenos presupuesto" os llega como nombre, email, teléfono, asunto y mensaje. Los días que se van en entender qué quiere el cliente antes de presupuestar también cuentan en el plazo. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/tres-i-tres
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: reformas e interiorismo. El formulario lleva reCAPTCHA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="165" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Reformas Escrivá Sanjuan</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>comercial@escrivasanjuan.com</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>https://escrivasanjuan.com/contacto</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>http://www.escrivasanjuan.com</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/escriva-sanjuan</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas Escrivá Sanjuan:
+Lleváis más de 35 años haciendo reformas en Gandia y la Safor y ofrecéis presupuesto sin compromiso, pero el formulario pregunta nombre, email, teléfono y asunto, y nada de la reforma. Todo lo que determina el presupuesto lo averiguáis después. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada solicitud ya explicada:
+https://presupuestos.nico-soto.es/demo/escriva-sanjuan
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. También tiene WhatsApp (+34 607 64 14 32), por si el formulario falla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="165" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>M&amp;A Instaladores</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>tecnicoacustermic@gmail.com</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>https://myainstaladores.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>https://myainstaladores.com</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/mya-instaladores</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de M&amp;A Instaladores:
+Hacéis pladur, aislamiento y reformas integrales, y la web le pide al cliente que os "cuente su proyecto" en un mensaje. Luego sois vosotros los que tenéis que traducir ese texto a metros, trabajos y presupuesto antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros ya estructurado:
+https://presupuestos.nico-soto.es/demo/mya-instaladores
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: pladur y aislamientos además de reformas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="165" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Vimoa</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>vicente@vimoa.es</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>https://vimoa.es/contacto</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>http://www.vimoa.es</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/vimoa</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Vimoa:
+Vuestro formulario de contacto pide solo un email y un mensaje, ni siquiera un teléfono. Y hacéis de todo, desde carpintería y armarios hasta reformas integrales, así que cada solicitud empieza con varios correos de ida y vuelta para saber qué quiere el cliente. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/vimoa
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="n"/>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. El formulario lleva reCAPTCHA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="165" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>DLUXE Solutions · Reformas en Oliva</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>info@reformasenoliva.es</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>https://reformasenoliva.es/</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>https://reformasenoliva.es</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/dluxesolutions</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de DLUXE Solutions:
+Vuestra web dice "solicita tu presupuesto y sorpréndete con el precio", pero el formulario solo recoge nombre, email, teléfono, código postal y qué tipo de reforma quiere. La sorpresa llega después de llamar, medir y preparar el presupuesto. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada, con metros, alcance, plazo e inversión:
+https://presupuestos.nico-soto.es/demo/dluxesolutions
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. El formulario está en la home. Solo 6 reseñas. También tiene WhatsApp (+34 679 37 36 75).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="165" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Construcciones y Reformas Salvicar</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>salvicar@ono.com</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>https://reformas.salvicar.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>http://www.salvicar.com</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/salvicar</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Salvicar:
+Vuestra web dice "Por fin, tenemos la solución para tus reformas" y que personalizáis cada proyecto y presupuesto. Pero para pedirlo, el cliente solo puede dejar nombre, email y un mensaje, después de resolver un captcha. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/salvicar
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="n"/>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. El formulario lleva un código antispam de Jimdo que hay que teclear a mano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="165" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>ObraEstil</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>obraestil@gmail.com</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>https://obraestil.es/contact/</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>http://www.obraestil.es</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/obraestil</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de ObraEstil:
+Os presentáis como especialistas en revestimientos, cocinas y baños, pero el formulario pide nombre, email, asunto y mensaje, sin teléfono ni nada de la obra. Cada solicitud empieza escribiendo al cliente para preguntarle lo básico. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/obraestil
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Entra por Gala Projectes, que se cae: es almacén y tienda de materiales de carpintería, no empresa de reformas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(prospeccion): lote 4 con las demos verificadas en el Excel
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -3747,7 +3747,7 @@
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: estudio de arquitectura que hace reformas íntegras de vivienda y locales (56 reseñas, 4,9).</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. Clase B: estudio de arquitectura que hace reformas íntegras de vivienda y locales (56 reseñas, 4,9).</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="J3" s="9" t="n"/>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: constructora y estudio de arquitectura, con obra nueva además de reformas.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. Clase B: constructora y estudio de arquitectura, con obra nueva además de reformas.</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3859,7 @@
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: estudio de interiorismo. El formulario está al pie de la home (email y un campo más) y lleva reCAPTCHA; la página «Contacta con nosotros» no tiene formulario.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. Clase B: estudio de interiorismo. El formulario está al pie de la home (email y un campo más) y lleva reCAPTCHA; la página «Contacta con nosotros» no tiene formulario.</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       <c r="J5" s="9" t="n"/>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. El formulario está al final de la home (no hay página de contacto aparte). El email de su ficha es de otro dominio (construccionesoliver.es): usa el formulario.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. El formulario está al final de la home (no hay página de contacto aparte). El email de su ficha es de otro dominio (construccionesoliver.es): usa el formulario.</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Hacen también obra nueva, locales y naves: la reforma de vivienda es una parte.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. Hacen también obra nueva, locales y naves: la reforma de vivienda es una parte.</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       <c r="J7" s="9" t="n"/>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: cocinas, armarios y carpintería a medida más que reforma integral. El formulario lleva reCAPTCHA.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. Clase B: cocinas, armarios y carpintería a medida más que reforma integral. El formulario lleva reCAPTCHA.</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       <c r="J8" s="4" t="n"/>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. No tiene email en la ficha. También tiene WhatsApp en la web, por si el formulario falla.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. No tiene email en la ficha. También tiene WhatsApp en la web, por si el formulario falla.</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4135,7 @@
       <c r="J9" s="9" t="n"/>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: interiorismo y carpintería a medida con reformas. El email de su ficha es de relleno (contacto@ejemplo.com); el real de su web es info@mesform.es. Usa el formulario.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. Clase B: interiorismo y carpintería a medida con reformas. El email de su ficha es de relleno (contacto@ejemplo.com); el real de su web es info@mesform.es. Usa el formulario.</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       <c r="J10" s="4" t="n"/>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: reformas e interiorismo. El formulario lleva reCAPTCHA.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. Clase B: reformas e interiorismo. El formulario lleva reCAPTCHA.</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       <c r="J11" s="9" t="n"/>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. También tiene WhatsApp (+34 607 64 14 32), por si el formulario falla.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. También tiene WhatsApp (+34 607 64 14 32), por si el formulario falla.</t>
         </is>
       </c>
     </row>
@@ -4303,7 +4303,7 @@
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Clase B: pladur y aislamientos además de reformas.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. Clase B: pladur y aislamientos además de reformas.</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4359,7 @@
       <c r="J13" s="9" t="n"/>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. El formulario lleva reCAPTCHA.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. El formulario lleva reCAPTCHA.</t>
         </is>
       </c>
     </row>
@@ -4415,7 +4415,7 @@
       <c r="J14" s="4" t="n"/>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. El formulario está en la home. Solo 6 reseñas. También tiene WhatsApp (+34 679 37 36 75).</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. El formulario está en la home. Solo 6 reseñas. También tiene WhatsApp (+34 679 37 36 75).</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       <c r="J15" s="9" t="n"/>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. El formulario lleva un código antispam de Jimdo que hay que teclear a mano.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. El formulario lleva un código antispam de Jimdo que hay que teclear a mano.</t>
         </is>
       </c>
     </row>
@@ -4527,7 +4527,7 @@
       <c r="J16" s="4" t="n"/>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>Demo pendiente de verificar. Formulario verificado 13/09 en Chrome. Entra por Gala Projectes, que se cae: es almacén y tienda de materiales de carpintería, no empresa de reformas.</t>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 en Chrome. Entra por Gala Projectes, que se cae: es almacén y tienda de materiales de carpintería, no empresa de reformas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(prospeccion): enlaces heredados en las hojas de los lotes 3 y 4 del Excel
Al copiar la hoja del lote anterior se quedaban sus hipervínculos: email,
formulario, web y demo apuntaban a empresas del lote 2 aunque el texto era el
correcto. Quitados en las hojas 2, 3 y 4.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -544,7 +544,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -573,7 +572,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
@@ -595,7 +593,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -617,7 +614,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -639,7 +635,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -2553,67 +2548,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L16"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId59"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2887,11 +2821,7 @@
           <t>8.0</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>mailto:hola@azaharreformasvalencia.com</t>
-        </is>
-      </c>
+      <c r="D5" s="10" t="n"/>
       <c r="E5" s="10" t="inlineStr">
         <is>
           <t>https://www.reformasvilla.com/contacto/</t>
@@ -3055,11 +2985,7 @@
           <t>7.5</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>mailto:info@obrasvip.com</t>
-        </is>
-      </c>
+      <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
           <t>https://wa.me/34650408834</t>
@@ -3545,67 +3471,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L16"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId59"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4533,67 +4398,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L16"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId59"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(prospeccion): Madrid 1 en la cola, para enviar a la vez que el lote 2
Búsqueda en 18 municipios del sur y el este de Madrid (196 empresas con web),
auditoría de 194 (77 A, 70 B, 47 C) guardada en events con lote madrid-1.
Los 15 mejores A con formulario revisado en Chrome y citas comprobadas contra
su web: mensajes en la cola, CSV, hoja en el Excel y documento del lote.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/prospeccion/cola-envio-home-estimator.xlsx
+++ b/docs/prospeccion/cola-envio-home-estimator.xlsx
@@ -10,14 +10,15 @@
     <sheet name="Leeme" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Lote 1 (1-15) enviado" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Lote 2 (16-30)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lote 3 (31-45)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Lote 4 (46-60)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Madrid 1 (61-75)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lote 3 (31-45)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Lote 4 (46-60)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lote 1 (1-15) enviado'!$A$1:$L$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lote 2 (16-30)'!$A$1:$L$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lote 3 (31-45)'!$A$1:$L$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Lote 4 (46-60)'!$A$1:$L$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Lote 3 (31-45)'!$A$1:$L$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Lote 4 (46-60)'!$A$1:$L$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -531,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -540,7 +541,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cola de envio Home Estimator - reformas Valencia</t>
+          <t>Cola de envio Home Estimator - reformas Valencia y Madrid</t>
         </is>
       </c>
     </row>
@@ -572,71 +573,78 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Hoja 'Madrid 1 (61-75)': 15 pendientes, montado el 13/09 (sur y este de Madrid, auditoría de 194 webs). Enviar EL MISMO DIA que el lote 2 para comparar zonas. Varada, Iasa Design y Foydecor tienen mas estructura de marketing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>Enlace de la demo</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Cada lead tiene su preview de marca en https://presupuestos.nico-soto.es/demo/&lt;slug&gt;,</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Cada lead tiene su preview de marca en https://presupuestos.nico-soto.es/demo/&lt;slug&gt;,</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>con su logo y sus colores. Verificado el 12/09: las 15 del lote 2 responden 200.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Datos para rellenar los formularios</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Email de respuesta:  hola@nico-soto.es</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Email de respuesta:  hola@nico-soto.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Telefono / WhatsApp: +34 600 78 22 11</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Lead 25 (REFORMSPEED) no tiene email y su web da error 500: se contacta por WhatsApp manual al +34 631 02 90 72 (Google Maps)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lead 23 (BONO PROYECTOS): el email tiene errata, usar el formulario.</t>
+          <t>Lead 25 (REFORMSPEED) no tiene email y su web da error 500: se contacta por WhatsApp manual al +34 631 02 90 72 (Google Maps)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Lead 23 (BONO PROYECTOS): el email tiene errata, usar el formulario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>'Demo abierta' sale de la analítica del proyecto Lovable reform-wizard (visitas 25/08-12/09; pueden incluir pruebas propias).</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Lead 37 (Estil Nou Miravet) no tiene formulario ni email: WhatsApp manual al +34 650 40 88 34.</t>
         </is>
@@ -2638,14 +2646,12 @@
       </c>
     </row>
     <row r="2" ht="165" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="A2" s="3" t="n">
+        <v>61</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Renovat Reformas</t>
+          <t>Reformas Blancor · Alcorcón</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
@@ -2655,29 +2661,29 @@
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>info@reformasrenovat.com</t>
+          <t>info@reformasblancor.es</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>https://www.reformasrenovat.com/</t>
+          <t>https://reformasblancor.es/presupuesto-para-reforma-integral-en-madrid/</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>http://www.reformasrenovat.com</t>
+          <t>https://reformasblancor.es</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>https://presupuestos.nico-soto.es/demo/renovat-reformas</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-blancor</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Hola, equipo de Renovat Reformas:
-He visto vuestro bloque de "Pide presupuesto sin compromiso": seis campos obligatorios (nombre, apellidos, email, teléfono, asunto y mensaje) y ninguno pregunta por la reforma. Con casi 150 reseñas, cada solicitud que entra todavía os obliga a averiguar metros, estancias e inversión antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros ya explicada:
-https://presupuestos.nico-soto.es/demo/renovat-reformas
+          <t>Hola, equipo de Reformas Blancor:
+En vuestra página de presupuesto explicáis que el coste de una reforma integral varía según los metros cuadrados de la vivienda, la calidad de los materiales y la complejidad de la redistribución. Pero el formulario solo pide nombre, email, teléfono y un mensaje opcional, así que todo eso lo tenéis que averiguar vosotros después, llamada a llamada. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma con esos datos ya contestados:
+https://presupuestos.nico-soto.es/demo/reformas-blancor
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
@@ -2689,107 +2695,99 @@
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). El formulario está en la home, en el bloque «Pide presupuesto sin compromiso» (no hay página de contacto aparte).</t>
+          <t>Demo verificada 13/09 (200, con su nombre). Formulario sin captcha. 174 reseñas (4,8).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="165" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Reformas y Pintores Nico</t>
+      <c r="A3" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Varada Reformas · Torrejón de Ardoz</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>pintoresnico@gmail.com</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>https://xn--reformaypintoresnicoespaa-woc.com/es</t>
-        </is>
-      </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>https://xn--reformaypintoresnicoespaa-woc.com</t>
-        </is>
-      </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>https://presupuestos.nico-soto.es/demo/reformas-pintores-nico</t>
-        </is>
-      </c>
-      <c r="H3" s="11" t="inlineStr">
-        <is>
-          <t>Hola, equipo de Reformas y Pintores Nico:
-Con más de 500 reseñas, imagino que os entra de todo. Por el mismo formulario de nombre, email, teléfono y mensaje os llega igual pintar un salón que una reforma integral, y no lo sabéis hasta que llamáis. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada solicitud ya separada y explicada:
-https://presupuestos.nico-soto.es/demo/reformas-pintores-nico
-Son solo dos minutos y sin compromiso.</t>
-        </is>
-      </c>
-      <c r="I3" s="11" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J3" s="9" t="n"/>
-      <c r="K3" s="11" t="inlineStr">
-        <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). El formulario está en la home y lleva reCAPTCHA. Mezcla reformas con pintura y comunidades: si se trata como B, su score baja a ~7,5.</t>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>https://varada.es/</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>https://varada.es</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/varada</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Varada:
+Prometéis "Respuesta en menos de 24h" y "Presupuesto cerrado", pero el formulario solo pide nombre, email, asunto y mensaje. Esas 24 horas empiezan con una llamada para saber qué quiere reformar el cliente, cuántos metros tiene y con qué presupuesto cuenta. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/varada
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="n"/>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su nombre). Empresa con más estructura: fichas en Madrid y Guadalajara con enlaces de campaña en Google. Es de las que más propuestas reciben. El formulario lleva reCAPTCHA. Sin email en la ficha: usa el formulario.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="165" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="A4" s="3" t="n">
+        <v>63</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Mestre Reformas</t>
+          <t>Raynadecor · Móstoles</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>info@mestrereformas.com</t>
+          <t>info@raynadecor.es</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>https://www.mestrereformas.com/contacto/</t>
+          <t>https://raynadecor.es/contacto/</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>https://www.mestrereformas.com</t>
+          <t>https://raynadecor.es</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>https://presupuestos.nico-soto.es/demo/mestre-reformas</t>
+          <t>https://presupuestos.nico-soto.es/demo/raynadecor</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Hola, equipo de Mestre Reformas:
-Prometéis precios cerrados y presupuesto en menos de 48 horas, pero el formulario de contacto solo pide nombre, correo y mensaje: ni teléfono, ni metros, ni qué estancia. Para cumplir esas 48 horas, lo primero es perseguir al cliente para saber qué quiere. He montado una demo con vuestra marca para enseñaros cómo podría llegaros la reforma ya explicada:
-https://presupuestos.nico-soto.es/demo/mestre-reformas
+          <t>Hola, equipo de Raynadecor:
+Vuestra web dice "Calculamos tu Presupuesto sin Compromiso" y que cada cliente recibirá un presupuesto personalizado. Pero para calcularlo, el formulario solo os deja nombre, email, teléfono y un mensaje: qué reforma es, cuántos metros tiene y con cuánto cuenta lo tenéis que preguntar después. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/raynadecor
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
@@ -2801,103 +2799,99 @@
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Su botón «Solicita tu presupuesto Gratis» de la home es solo un enlace de teléfono: el formulario está en /contacto.</t>
+          <t>Demo verificada 13/09 (200, con su nombre). El formulario lleva reCAPTCHA.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="165" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Reformas Villa</t>
+      <c r="A5" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Construcciones J.D.M. · Alcobendas</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>8.0</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>https://www.reformasvilla.com/contacto/</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>http://www.reformasvilla.com</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>https://presupuestos.nico-soto.es/demo/reformas-villa</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>Hola, equipo de Reformas Villa:
-Vuestros proyectos son pisos completos, reformas integrales, cocinas y baños, pero por la web solo os llega un nombre, un email y un mensaje. Cada solicitud os obliga a empezar preguntando lo básico antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma con metros, estancias, plazo e inversión ya recogidos:
-https://presupuestos.nico-soto.es/demo/reformas-villa
-Son solo dos minutos y sin compromiso.</t>
-        </is>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J5" s="9" t="n"/>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>https://construccionesjdm.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>https://construccionesjdm.com</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/construcciones-jdm</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Construcciones J.D.M.:
+Vuestra página de contacto se llama "Pide ya tu presupuesto" y promete un presupuesto personalizado para cada reforma, pero el formulario pide nombre, apellidos, teléfono, email, asunto y mensaje: nada de la vivienda ni de la obra. Lo personalizado empieza después, preguntando lo básico. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/construcciones-jdm
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su nombre). El formulario lleva reCAPTCHA. Sin email en la ficha: usa el formulario.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="165" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="A6" s="3" t="n">
+        <v>65</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Macamon Reformas Integrales</t>
+          <t>Reformas Integrales Areal · Alcorcón</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>macamoncho@gmail.com</t>
+          <t>arealsl@arealsl.es</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>https://macamoncho.es/presupuestos/</t>
+          <t>https://reformasintegralesareal.es/contacto-reformas-integral-madrid</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>http://macamoncho.es</t>
+          <t>https://reformasintegralesareal.es</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>https://presupuestos.nico-soto.es/demo/macamon-reformas</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-areal</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Hola, equipo de Macamon Reformas:
-Vuestra página "Pide tu presupuesto a medida" ya pregunta qué necesita el cliente y para dónde, que es más de lo que hace casi todo el sector. Pero lo recoge en texto libre: ni metros, ni plazo, ni con cuánto cuenta. He preparado una demo con vuestra marca para completar justo esa parte:
-https://presupuestos.nico-soto.es/demo/macamon-reformas
+          <t>Hola, equipo de Reformas Areal:
+En vuestra página de contacto ofrecéis presupuesto sin compromiso y responder lo antes posible, pero el formulario solo recoge nombre, email, teléfono y un mensaje. Antes de poder contestar con algo concreto os toca preguntar los metros, las estancias y cuándo quiere empezar el cliente. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/reformas-areal
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
@@ -2909,103 +2903,99 @@
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Lleva reCAPTCHA v3 (invisible): no debería pedirte nada, pero si el envío falla, prueba desde otro navegador.</t>
+          <t>Demo verificada 13/09 (200, con su nombre). Formulario sin captcha.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="165" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Hidro2 Grup</t>
+      <c r="A7" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Quality Reform · Fuenlabrada</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>7.5</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>info@hidro2grup.com</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>https://www.hidro2grup.com/contacto/</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>https://www.hidro2grup.com</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>https://presupuestos.nico-soto.es/demo/hidro2-grup</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>Hola, equipo de Hidro2 Grup:
-En vuestra web un cliente cuenta que fuisteis a medir en 48 horas y tuvo el presupuesto detallado en una semana. Es muy buen servicio, pero el formulario (nombre, email, teléfono y mensaje) no adelanta nada de esa semana: todo empieza cuando ya ha llegado el lead. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado antes de desplazaros:
-https://presupuestos.nico-soto.es/demo/hidro2-grup
-Son solo dos minutos y sin compromiso.</t>
-        </is>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J7" s="9" t="n"/>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>http://qualityreform.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>https://qualityreform.com</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/quality-reform</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Quality Reform:
+Vuestra página de contacto dice "Pide presupuesto sin compromiso" y pide rellenar el formulario, pero el formulario solo recoge los datos de contacto y un comentario. Hacéis desde reformas integrales hasta pequeñas reparaciones, y por ahí os entra todo igual hasta que habláis con el cliente. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/quality-reform
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="n"/>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su nombre). El formulario lleva Turnstile de Cloudflare (casilla de verificación). Sin email en la ficha. También tiene WhatsApp (+34 643 85 91 35).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="165" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
+      <c r="A8" s="3" t="n">
+        <v>67</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Estil Nou Miravet</t>
+          <t>Iasa Design · Rivas-Vaciamadrid</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>7.5</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n"/>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>contacto@iasadesign.com</t>
+        </is>
+      </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>https://wa.me/34650408834</t>
+          <t>https://www.iasadesign.com/contacto/</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>https://estilnoumiravet.com</t>
+          <t>https://www.iasadesign.com</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>https://presupuestos.nico-soto.es/demo/estil-nou-miravet</t>
+          <t>https://presupuestos.nico-soto.es/demo/iasa-design</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Hola, equipo de Estil Nou Miravet:
-He visto que vuestro botón "Solicitar presupuesto" abre directamente un WhatsApp. Eso hace que cada reforma empiece con una conversación desde cero: qué quiere hacer, metros, estancias, plazo e inversión, antes de saber siquiera si merece la pena. He montado una demo con vuestra marca para que todo eso os llegue recogido antes de empezar a hablar:
-https://presupuestos.nico-soto.es/demo/estil-nou-miravet
+          <t>Hola, equipo de Iasa Design:
+Ya publicáis promociones con precio, desde 4.850 € un baño hasta 29.850 € una integral, así que quien os escribe quiere una cifra pronto. Pero al pulsar "Pedir presupuesto sin compromiso" llega a un formulario de nombre, email, teléfono y mensaje, sin decir qué quiere reformar ni cuántos metros tiene. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/iasa-design
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
@@ -3017,107 +3007,103 @@
       <c r="J8" s="4" t="n"/>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Demo verificada 13/09 (200, con su logo). Por WhatsApp (sin formulario). Por WhatsApp, no por formulario: no tiene formulario ni email; todos los «Solicitar presupuesto» de su web abren WhatsApp. El enlace abre WhatsApp con su móvil (+34 650 40 88 34). Pega el mismo mensaje, a mano.</t>
+          <t>Demo verificada 13/09 (200, con su nombre). Marketing más trabajado (promociones con precio, Kit Digital): de las que más propuestas reciben. El formulario lleva reCAPTCHA. Logo blanco: la demo usa una versión sobre fondo oscuro (iasa-design-fondo.png).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="165" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Reformas Antoine</t>
+      <c r="A9" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Reformas Foydecor · Móstoles</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>7.5</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>nikolaytsverkov@gmail.com</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>https://reformasytrasterosantuine.com/es</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>https://reformasytrasterosantuine.com</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>https://presupuestos.nico-soto.es/demo/reformas-antoine</t>
-        </is>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>Hola, equipo de Reformas Antoine:
-Hacéis desde pequeñas reparaciones hasta reformas completas, y las dos os llegan por el mismo formulario de nombre, email, teléfono y mensaje. Hasta que no habláis con el cliente no sabéis si es un arreglo de una tarde o una obra de dos meses. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada solicitud ya explicada:
-https://presupuestos.nico-soto.es/demo/reformas-antoine
-Son solo dos minutos y sin compromiso.</t>
-        </is>
-      </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J9" s="9" t="n"/>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Clase B: además de reformas alquila trasteros. El formulario está en la home y lleva reCAPTCHA.</t>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>foydecor@gmail.com</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>https://foydecor.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>https://foydecor.com</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/foydecor</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Foydecor:
+Prometéis proyectos adaptados a las necesidades de cada cliente "y, como no, a su presupuesto", y además financiáis sin intereses. Pero el formulario pide nombre, correo, teléfono, asunto y "Escriba aquí su consulta": con cuánto cuenta el cliente y qué quiere reformar lo tenéis que preguntar después. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/foydecor
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="n"/>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su nombre). Hacen anuncio en Telemadrid: empresa con más estructura. El formulario lleva reCAPTCHA.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="165" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
+      <c r="A10" s="3" t="n">
+        <v>69</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Reformas integrales Cuinex</t>
+          <t>Reformas El Baúl · Móstoles</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>info@cuinexreformas.es</t>
+          <t>elbaul@reformaselbaul.com</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>https://www.cuinexreformas.es/contacto</t>
+          <t>https://www.reformaselbaul.com/contacto/</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>http://www.cuinexreformas.es</t>
+          <t>https://www.reformaselbaul.com</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>https://presupuestos.nico-soto.es/demo/cuinex</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-el-baul</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Hola, equipo de Cuinex:
-Me llamó la atención que vuestro formulario pida el DNI o NIF del cliente, pero no qué quiere reformar ni cuántos metros tiene. Sabéis quién es antes de saber si el proyecto merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
-https://presupuestos.nico-soto.es/demo/cuinex
+          <t>Hola, equipo de Reformas El Baúl:
+Vuestra web dice "Llámenos y le daremos el mejor presupuesto", pero quien prefiere escribir llega a un formulario de nombre, email, teléfono y mensaje. Sin saber qué quiere reformar ni cuántos metros tiene, ese mejor presupuesto empieza con varias llamadas. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/reformas-el-baul
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
@@ -3129,107 +3115,103 @@
       <c r="J10" s="4" t="n"/>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Clase B: tira mucho a cocinas y carpintería. El formulario pregunta si eres particular o empresa y pide DNI/NIF.</t>
+          <t>Demo verificada 13/09 (200, con su nombre). El formulario lleva reCAPTCHA. También tiene WhatsApp (+34 656 68 48 85).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="165" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Jesbal Habitatge</t>
+      <c r="A11" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Reformas AlcoMad · Alcorcón</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>7.0</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>info@jesbalhabitatge.es</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>https://jesbalhabitatge.es/contacto/</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>https://jesbalhabitatge.es</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>https://presupuestos.nico-soto.es/demo/jesbal-habitatge</t>
-        </is>
-      </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>Hola, equipo de Jesbal Habitatge:
-Vuestra web ya explica que una integral de unos 100 m² lleva 2-3 meses y que ayudáis con la financiación, pero el formulario solo pregunta el tipo de reforma: ni metros, ni plazo, ni inversión. Justo lo que sabéis explicar tan bien es lo que no llega en la solicitud. He montado una demo con vuestra marca para enseñaros cómo podría llegaros ya completa:
-https://presupuestos.nico-soto.es/demo/jesbal-habitatge
-Son solo dos minutos y sin compromiso.</t>
-        </is>
-      </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="n"/>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>contacto@reformasalcomad.es</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>https://www.reformasalcomad.es/</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>https://www.reformasalcomad.es</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-alcomad</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de AlcoMad:
+Vuestro formulario ya pregunta si es reforma integral, cocina, baño o local, que es más de lo que pregunta la mayoría. Pero después de "¡Solicite presupuesto sin compromiso!" seguís sin saber los metros, las calidades ni cuándo quiere empezar el cliente, y eso sale en la primera llamada. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/reformas-alcomad
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="n"/>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su nombre). El formulario está en la home, sin captcha.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="165" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
+      <c r="A12" s="3" t="n">
+        <v>71</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Gytech group</t>
+          <t>Reformas Marian · Torrejón de Ardoz</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>info@gytechgroup.com</t>
+          <t>hola@reformasmarian.es</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>https://gytechgroup.com/contacto/</t>
+          <t>https://reformasmarian.es/contacto/</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>https://gytechgroup.com</t>
+          <t>https://reformasmarian.es</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>https://presupuestos.nico-soto.es/demo/gytech-group</t>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-marian</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Hola, equipo de Gytech:
-Ofrecéis presupuesto sin compromiso, pero hasta saber si el proyecto es real el compromiso lo ponéis vosotros: llamadas, desplazamiento, medición y horas de presupuesto. Y el formulario solo recoge nombre, email, teléfono, asunto y mensaje. He montado una demo con vuestra marca para enseñaros cómo entender el proyecto antes de dedicarle ese tiempo:
-https://presupuestos.nico-soto.es/demo/gytech-group
+          <t>Hola, equipo de Reformas Marian:
+En vuestra página de contacto invitáis a "pedir un presupuesto sin compromiso", pero el formulario solo pide nombre, email, móvil y mensaje. Hasta que no habláis con el cliente no sabéis si es un baño, una cocina o un piso entero, ni cuántos metros tiene. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/reformas-marian
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
@@ -3241,107 +3223,103 @@
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+          <t>Demo verificada 13/09 (200, con su nombre). El formulario lleva reCAPTCHA. Su web no tiene logo en imagen (nombre en texto): la demo compone el nombre con su amarillo.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="165" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Construcciones y Reformas Génesis</t>
+      <c r="A13" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Support Home · Valdemoro</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>6.5</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>contacto@reformasgenesis.com.es</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>https://www.reformasgenesis.com.es/</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>http://www.reformasgenesis.com.es</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>https://presupuestos.nico-soto.es/demo/reformas-genesis</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>Hola, equipo de Reformas Génesis:
-Hacéis de todo, desde un baño o una cocina hasta una reforma integral, una piscina o una nave, y por la web os llega igual: nombre, email y un mensaje. Hasta que no habláis con el cliente no sabéis cuál de todas es ni si merece la pena el desplazamiento. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
-https://presupuestos.nico-soto.es/demo/reformas-genesis
-Son solo dos minutos y sin compromiso.</t>
-        </is>
-      </c>
-      <c r="I13" s="11" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J13" s="9" t="n"/>
-      <c r="K13" s="11" t="inlineStr">
-        <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Entra por Aquí tu Reforma, que se cae: es una cadena nacional con tiendas y franquicias y ya tiene su propio formulario de presupuesto de 7 pasos. El formulario está en la home, al final (nombre, email, mensaje). También tiene WhatsApp (+34 613 36 88 72) por si falla.</t>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>servicios@supporthome.es</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>https://supporthome.es/contacto/</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>https://supporthome.es</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/support-home</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Support Home:
+Decís que entregáis el presupuesto "con total transparencia en cuanto a materiales, mano de obra y tiempo de ejecución", pero para pedirlo el formulario solo recoge nombre, email, teléfono, asunto y un mensaje. Esa transparencia empieza después de preguntarle al cliente qué quiere reformar y cuántos metros tiene. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/support-home
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su nombre). Reformas y servicios (algo de multiservicio). reCAPTCHA invisible. También tiene WhatsApp (667 93 95 11).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="165" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
+      <c r="A14" s="3" t="n">
+        <v>73</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Reformas y Proyectos Sacaber</t>
+          <t>Remacen Reparaciones · Alcalá de Henares</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>sacaber@hotmail.com</t>
+          <t>reformasmadridcentro@gmail.com</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>http://sacaber.com/contacto</t>
+          <t>https://www.reformasmadridcentro.com/contacto</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>http://sacaber.com</t>
+          <t>https://www.reformasmadridcentro.com</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>https://presupuestos.nico-soto.es/demo/sacaber</t>
+          <t>https://presupuestos.nico-soto.es/demo/remacen</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Hola, equipo de Reformas Sacaber:
-He visto que vuestro formulario recoge nombre, email, teléfono y un mensaje, y poco más. Es decir, todo el trabajo de entender la reforma (metros, estancias, alcance, inversión) empieza cuando ya ha llegado el lead. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado:
-https://presupuestos.nico-soto.es/demo/sacaber
+          <t>Hola, equipo de Remacen:
+En vuestra web ofrecéis presupuesto gratuito y respuesta rápida, pero el formulario pide nombre, apellidos, email, teléfono y mensaje, sin nada de la obra. Esa respuesta rápida empieza preguntando lo básico: qué reforma es, cuántos metros tiene y con qué presupuesto cuenta el cliente. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/remacen
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
@@ -3353,107 +3331,99 @@
       <c r="J14" s="4" t="n"/>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+          <t>Demo verificada 13/09 (200, con su nombre). reCAPTCHA invisible. Su web no tiene logo en imagen: la demo compone el nombre con su dorado. También tiene WhatsApp (+34 601 23 84 93).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="165" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Construcciones y Reformas Ramírez Castañeda</t>
+      <c r="A15" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Reformas Vegam · Alcobendas</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>6.5</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>ramirezcastanedasl@gmail.com</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>https://www.xn--construccionesyreformasramirezcastaedasl-n2d.es/contactanos</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>http://xn--construccionesyreformasramirezcastaedasl-n2d.es</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>https://presupuestos.nico-soto.es/demo/ramirez-castaneda</t>
-        </is>
-      </c>
-      <c r="H15" s="11" t="inlineStr">
-        <is>
-          <t>Hola, equipo de Construcciones y Reformas Ramírez Castañeda:
-He visto que en vuestra página de contacto el cliente os deja sus datos y un mensaje libre. Todo lo que determina el presupuesto (qué quiere reformar, metros, plazo e inversión) tenéis que sacarlo después, llamada a llamada. He preparado una demo con vuestra marca para enseñaros cómo podría llegaros ya recogido:
-https://presupuestos.nico-soto.es/demo/ramirez-castaneda
-Son solo dos minutos y sin compromiso.</t>
-        </is>
-      </c>
-      <c r="I15" s="11" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J15" s="9" t="n"/>
-      <c r="K15" s="11" t="inlineStr">
-        <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>https://www.reformasvegam.es/contacto</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>https://www.reformasvegam.es</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-vegam</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas Vegam:
+Entre lo que os distingue ponéis "Presupuestos sin compromiso" y "Claridad total desde el primer momento". Pero ese primer momento es un formulario de nombre, email, teléfono y mensaje, y la claridad llega después, cuando ya habéis preguntado qué quiere reformar el cliente y cuántos metros tiene. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/reformas-vegam
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="n"/>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su nombre). reCAPTCHA invisible. El email de su ficha es personal (hotmail): usa el formulario. También tiene WhatsApp (+34 659 20 10 03).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="165" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="A16" s="3" t="n">
+        <v>75</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Multiservicios AM Levante</t>
+          <t>Grupo León Reformas · Getafe</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>multiserviciosam375@gmail.com</t>
+          <t>grupoleon.gerencia.getafe@gmail.com</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>https://www.multiserviciosamlevante.es/contactanos</t>
+          <t>https://grupoleonreformas.com/contacto/</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>http://www.multiserviciosamlevante.es</t>
+          <t>https://grupoleonreformas.com</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>https://presupuestos.nico-soto.es/demo/multiservicios-am-levante</t>
+          <t>https://presupuestos.nico-soto.es/demo/grupo-leon-reformas</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Hola, equipo de Multiservicios AM Levante:
-Hacéis reformas integrales y ofrecéis presupuesto sin compromiso, pero hasta saber si el proyecto es real el compromiso lo ponéis vosotros: llamadas, visita, medición y preparar el presupuesto. Por la web solo os llegan unos datos y un mensaje. He montado una demo con vuestra marca para enseñaros cómo entender el proyecto antes de dedicarle ese tiempo:
-https://presupuestos.nico-soto.es/demo/multiservicios-am-levante
+          <t>Hola, equipo de Grupo León Reformas:
+Vuestro botón dice "Consigue Tu Presupuesto Sin Compromiso", pero el formulario pide nombre, email, teléfono e "Información", un campo libre. Cada solicitud os obliga a volver a preguntar qué quiere reformar el cliente, cuántos metros tiene y con qué presupuesto cuenta. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/grupo-leon-reformas
 Son solo dos minutos y sin compromiso.</t>
         </is>
       </c>
@@ -3465,12 +3435,11 @@
       <c r="J16" s="4" t="n"/>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). También tiene WhatsApp (+34 623 26 65 67), por si el formulario falla.</t>
+          <t>Demo verificada 13/09 (200, con su nombre). El formulario lleva Turnstile de Cloudflare. Su web no tiene logo en imagen: la demo va en tinta con el nombre compuesto.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3563,6 +3532,929 @@
     <row r="2" ht="165" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Renovat Reformas</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>info@reformasrenovat.com</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>https://www.reformasrenovat.com/</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>http://www.reformasrenovat.com</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/renovat-reformas</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Renovat Reformas:
+He visto vuestro bloque de "Pide presupuesto sin compromiso": seis campos obligatorios (nombre, apellidos, email, teléfono, asunto y mensaje) y ninguno pregunta por la reforma. Con casi 150 reseñas, cada solicitud que entra todavía os obliga a averiguar metros, estancias e inversión antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros ya explicada:
+https://presupuestos.nico-soto.es/demo/renovat-reformas
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="n"/>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). El formulario está en la home, en el bloque «Pide presupuesto sin compromiso» (no hay página de contacto aparte).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="165" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Reformas y Pintores Nico</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>pintoresnico@gmail.com</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>https://xn--reformaypintoresnicoespaa-woc.com/es</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>https://xn--reformaypintoresnicoespaa-woc.com</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-pintores-nico</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas y Pintores Nico:
+Con más de 500 reseñas, imagino que os entra de todo. Por el mismo formulario de nombre, email, teléfono y mensaje os llega igual pintar un salón que una reforma integral, y no lo sabéis hasta que llamáis. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada solicitud ya separada y explicada:
+https://presupuestos.nico-soto.es/demo/reformas-pintores-nico
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="n"/>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). El formulario está en la home y lleva reCAPTCHA. Mezcla reformas con pintura y comunidades: si se trata como B, su score baja a ~7,5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="165" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Mestre Reformas</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>info@mestrereformas.com</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.mestrereformas.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.mestrereformas.com</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/mestre-reformas</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Mestre Reformas:
+Prometéis precios cerrados y presupuesto en menos de 48 horas, pero el formulario de contacto solo pide nombre, correo y mensaje: ni teléfono, ni metros, ni qué estancia. Para cumplir esas 48 horas, lo primero es perseguir al cliente para saber qué quiere. He montado una demo con vuestra marca para enseñaros cómo podría llegaros la reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/mestre-reformas
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Su botón «Solicita tu presupuesto Gratis» de la home es solo un enlace de teléfono: el formulario está en /contacto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="165" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Reformas Villa</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>https://www.reformasvilla.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>http://www.reformasvilla.com</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-villa</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas Villa:
+Vuestros proyectos son pisos completos, reformas integrales, cocinas y baños, pero por la web solo os llega un nombre, un email y un mensaje. Cada solicitud os obliga a empezar preguntando lo básico antes de saber si merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma con metros, estancias, plazo e inversión ya recogidos:
+https://presupuestos.nico-soto.es/demo/reformas-villa
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="n"/>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="165" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Macamon Reformas Integrales</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>macamoncho@gmail.com</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>https://macamoncho.es/presupuestos/</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>http://macamoncho.es</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/macamon-reformas</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Macamon Reformas:
+Vuestra página "Pide tu presupuesto a medida" ya pregunta qué necesita el cliente y para dónde, que es más de lo que hace casi todo el sector. Pero lo recoge en texto libre: ni metros, ni plazo, ni con cuánto cuenta. He preparado una demo con vuestra marca para completar justo esa parte:
+https://presupuestos.nico-soto.es/demo/macamon-reformas
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Lleva reCAPTCHA v3 (invisible): no debería pedirte nada, pero si el envío falla, prueba desde otro navegador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="165" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Hidro2 Grup</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>info@hidro2grup.com</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>https://www.hidro2grup.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>https://www.hidro2grup.com</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/hidro2-grup</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Hidro2 Grup:
+En vuestra web un cliente cuenta que fuisteis a medir en 48 horas y tuvo el presupuesto detallado en una semana. Es muy buen servicio, pero el formulario (nombre, email, teléfono y mensaje) no adelanta nada de esa semana: todo empieza cuando ya ha llegado el lead. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado antes de desplazaros:
+https://presupuestos.nico-soto.es/demo/hidro2-grup
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="165" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Estil Nou Miravet</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>https://wa.me/34650408834</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>https://estilnoumiravet.com</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/estil-nou-miravet</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Estil Nou Miravet:
+He visto que vuestro botón "Solicitar presupuesto" abre directamente un WhatsApp. Eso hace que cada reforma empiece con una conversación desde cero: qué quiere hacer, metros, estancias, plazo e inversión, antes de saber siquiera si merece la pena. He montado una demo con vuestra marca para que todo eso os llegue recogido antes de empezar a hablar:
+https://presupuestos.nico-soto.es/demo/estil-nou-miravet
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Por WhatsApp (sin formulario). Por WhatsApp, no por formulario: no tiene formulario ni email; todos los «Solicitar presupuesto» de su web abren WhatsApp. El enlace abre WhatsApp con su móvil (+34 650 40 88 34). Pega el mismo mensaje, a mano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="165" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Reformas Antoine</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>nikolaytsverkov@gmail.com</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>https://reformasytrasterosantuine.com/es</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>https://reformasytrasterosantuine.com</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-antoine</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas Antoine:
+Hacéis desde pequeñas reparaciones hasta reformas completas, y las dos os llegan por el mismo formulario de nombre, email, teléfono y mensaje. Hasta que no habláis con el cliente no sabéis si es un arreglo de una tarde o una obra de dos meses. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada solicitud ya explicada:
+https://presupuestos.nico-soto.es/demo/reformas-antoine
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="n"/>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Clase B: además de reformas alquila trasteros. El formulario está en la home y lleva reCAPTCHA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="165" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Reformas integrales Cuinex</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>info@cuinexreformas.es</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>https://www.cuinexreformas.es/contacto</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>http://www.cuinexreformas.es</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/cuinex</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Cuinex:
+Me llamó la atención que vuestro formulario pida el DNI o NIF del cliente, pero no qué quiere reformar ni cuántos metros tiene. Sabéis quién es antes de saber si el proyecto merece la pena. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/cuinex
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Clase B: tira mucho a cocinas y carpintería. El formulario pregunta si eres particular o empresa y pide DNI/NIF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="165" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Jesbal Habitatge</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>info@jesbalhabitatge.es</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>https://jesbalhabitatge.es/contacto/</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>https://jesbalhabitatge.es</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/jesbal-habitatge</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Jesbal Habitatge:
+Vuestra web ya explica que una integral de unos 100 m² lleva 2-3 meses y que ayudáis con la financiación, pero el formulario solo pregunta el tipo de reforma: ni metros, ni plazo, ni inversión. Justo lo que sabéis explicar tan bien es lo que no llega en la solicitud. He montado una demo con vuestra marca para enseñaros cómo podría llegaros ya completa:
+https://presupuestos.nico-soto.es/demo/jesbal-habitatge
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="165" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Gytech group</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>info@gytechgroup.com</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>https://gytechgroup.com/contacto/</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>https://gytechgroup.com</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/gytech-group</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Gytech:
+Ofrecéis presupuesto sin compromiso, pero hasta saber si el proyecto es real el compromiso lo ponéis vosotros: llamadas, desplazamiento, medición y horas de presupuesto. Y el formulario solo recoge nombre, email, teléfono, asunto y mensaje. He montado una demo con vuestra marca para enseñaros cómo entender el proyecto antes de dedicarle ese tiempo:
+https://presupuestos.nico-soto.es/demo/gytech-group
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="165" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Construcciones y Reformas Génesis</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>contacto@reformasgenesis.com.es</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>https://www.reformasgenesis.com.es/</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>http://www.reformasgenesis.com.es</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/reformas-genesis</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas Génesis:
+Hacéis de todo, desde un baño o una cocina hasta una reforma integral, una piscina o una nave, y por la web os llega igual: nombre, email y un mensaje. Hasta que no habláis con el cliente no sabéis cuál de todas es ni si merece la pena el desplazamiento. He montado una demo con vuestra marca para enseñaros cómo podría llegaros cada reforma ya explicada:
+https://presupuestos.nico-soto.es/demo/reformas-genesis
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="n"/>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). Entra por Aquí tu Reforma, que se cae: es una cadena nacional con tiendas y franquicias y ya tiene su propio formulario de presupuesto de 7 pasos. El formulario está en la home, al final (nombre, email, mensaje). También tiene WhatsApp (+34 613 36 88 72) por si falla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="165" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Reformas y Proyectos Sacaber</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>sacaber@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>http://sacaber.com/contacto</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>http://sacaber.com</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/sacaber</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Reformas Sacaber:
+He visto que vuestro formulario recoge nombre, email, teléfono y un mensaje, y poco más. Es decir, todo el trabajo de entender la reforma (metros, estancias, alcance, inversión) empieza cuando ya ha llegado el lead. He montado una demo con vuestra marca para enseñaros cómo podría llegaros el proyecto ya explicado:
+https://presupuestos.nico-soto.es/demo/sacaber
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="165" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Construcciones y Reformas Ramírez Castañeda</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>ramirezcastanedasl@gmail.com</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>https://www.xn--construccionesyreformasramirezcastaedasl-n2d.es/contactanos</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>http://xn--construccionesyreformasramirezcastaedasl-n2d.es</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/ramirez-castaneda</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Construcciones y Reformas Ramírez Castañeda:
+He visto que en vuestra página de contacto el cliente os deja sus datos y un mensaje libre. Todo lo que determina el presupuesto (qué quiere reformar, metros, plazo e inversión) tenéis que sacarlo después, llamada a llamada. He preparado una demo con vuestra marca para enseñaros cómo podría llegaros ya recogido:
+https://presupuestos.nico-soto.es/demo/ramirez-castaneda
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="n"/>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="165" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Multiservicios AM Levante</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>multiserviciosam375@gmail.com</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>https://www.multiserviciosamlevante.es/contactanos</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>http://www.multiserviciosamlevante.es</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>https://presupuestos.nico-soto.es/demo/multiservicios-am-levante</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Hola, equipo de Multiservicios AM Levante:
+Hacéis reformas integrales y ofrecéis presupuesto sin compromiso, pero hasta saber si el proyecto es real el compromiso lo ponéis vosotros: llamadas, visita, medición y preparar el presupuesto. Por la web solo os llegan unos datos y un mensaje. He montado una demo con vuestra marca para enseñaros cómo entender el proyecto antes de dedicarle ese tiempo:
+https://presupuestos.nico-soto.es/demo/multiservicios-am-levante
+Son solo dos minutos y sin compromiso.</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>Demo verificada 13/09 (200, con su logo). Formulario verificado 13/09 (200). También tiene WhatsApp (+34 623 26 65 67), por si el formulario falla.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L16"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>URL contacto</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Demo (URL)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje (listo para enviar)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Enviado</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha envio</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Demo abierta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="165" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
           <t>46</t>
         </is>
       </c>

</xml_diff>